<commit_message>
feat: integrate Fan Fest and Vive Tu Pasión campaigns with timebars and date fixes
</commit_message>
<xml_diff>
--- a/camino_cumbre/CAMINO A LA CUMBRE.xlsx
+++ b/camino_cumbre/CAMINO A LA CUMBRE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/camino_cumbre/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83244D24-AD13-8441-877F-9D70F7531BD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84CC8729-30BB-FB41-871F-6F3FD4BEAF7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="1500" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="42">
   <si>
     <t>Dir. de Venta</t>
   </si>
@@ -161,7 +161,7 @@
     <t>Pólizas Pagadas</t>
   </si>
   <si>
-    <t>Avance  al 28 de febrero de 2026.</t>
+    <t>Avance  al 11 de marzo de 2026.</t>
   </si>
 </sst>
 </file>
@@ -172,7 +172,7 @@
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -248,6 +248,26 @@
       <color indexed="12"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Bookshelf Symbol 7"/>
+      <family val="2"/>
+      <charset val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Bookshelf Symbol 7"/>
+      <family val="2"/>
+      <charset val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -393,7 +413,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -471,6 +491,11 @@
     <xf numFmtId="14" fontId="3" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="10" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -501,7 +526,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{5777CE91-9B5C-AD4F-B1FB-47F4B57F6892}"/>
     <cellStyle name="Porcentaje 2" xfId="2" xr:uid="{7B24C14E-EE44-314E-8590-6F0AEF4F900D}"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="24">
     <dxf>
       <border>
         <left style="hair">
@@ -542,171 +567,6 @@
         <extend val="0"/>
         <color indexed="10"/>
       </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -1024,7 +884,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X22" totalsRowShown="0" headerRowDxfId="32" headerRowBorderDxfId="31" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X22" totalsRowShown="0" headerRowDxfId="23" headerRowBorderDxfId="22" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
   <autoFilter ref="A4:X22" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}"/>
   <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{452BBEC3-C02A-954A-AF30-AAC8D4135219}" name="Dir. de Venta" dataCellStyle="Normal 2"/>
@@ -1033,21 +893,21 @@
     <tableColumn id="4" xr3:uid="{E64AD030-9FFA-1B49-B7F8-31458F00EB96}" name="Mat" dataCellStyle="Normal 2"/>
     <tableColumn id="5" xr3:uid="{407858BC-0878-5E44-A050-843285231653}" name="Suc" dataCellStyle="Normal 2"/>
     <tableColumn id="6" xr3:uid="{6FEB1162-A9E3-244F-886A-8D5C735D8BE4}" name="Asesor" dataCellStyle="Normal 2"/>
-    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="30" dataCellStyle="Normal 2"/>
-    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="29" dataCellStyle="Normal 2"/>
-    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="28" dataCellStyle="Porcentaje 2"/>
-    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="27" dataCellStyle="Normal 2"/>
-    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="26" dataCellStyle="Normal 2"/>
-    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="25" dataCellStyle="Normal 2"/>
-    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="24" dataCellStyle="Normal 2"/>
-    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="23" dataCellStyle="Normal 2"/>
-    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="22" dataCellStyle="Normal 2"/>
-    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="21" dataCellStyle="Normal 2"/>
-    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="20" dataCellStyle="Normal 2"/>
-    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="19" dataCellStyle="Normal 2"/>
-    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="18" dataCellStyle="Normal 2"/>
-    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="17" dataCellStyle="Normal 2"/>
-    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="16" dataCellStyle="Normal 2"/>
+    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="21" dataCellStyle="Normal 2"/>
+    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="20" dataCellStyle="Normal 2"/>
+    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="19" dataCellStyle="Porcentaje 2"/>
+    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="18" dataCellStyle="Normal 2"/>
+    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="17" dataCellStyle="Normal 2"/>
+    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="16" dataCellStyle="Normal 2"/>
+    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="15" dataCellStyle="Normal 2"/>
+    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="14" dataCellStyle="Normal 2"/>
+    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="13" dataCellStyle="Normal 2"/>
+    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="12" dataCellStyle="Normal 2"/>
+    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="11" dataCellStyle="Normal 2"/>
+    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="10" dataCellStyle="Normal 2"/>
+    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="9" dataCellStyle="Normal 2"/>
+    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="8" dataCellStyle="Normal 2"/>
+    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="7" dataCellStyle="Normal 2"/>
     <tableColumn id="22" xr3:uid="{FB6CEF72-668C-CB49-ACCA-75A997C036A1}" name="Mes 1" dataCellStyle="Normal 2"/>
     <tableColumn id="23" xr3:uid="{58B1F16B-3FBB-3D4C-8C16-DD05D985324B}" name="Mes 2" dataCellStyle="Normal 2"/>
     <tableColumn id="24" xr3:uid="{B5A4E59E-794B-AB4B-BB2B-840B78865464}" name="Mes 3" dataCellStyle="Normal 2"/>
@@ -1402,24 +1262,24 @@
       <c r="I3" s="7"/>
       <c r="J3" s="8"/>
       <c r="K3" s="9"/>
-      <c r="L3" s="36" t="s">
+      <c r="L3" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="M3" s="37"/>
-      <c r="N3" s="38"/>
-      <c r="P3" s="33" t="s">
+      <c r="M3" s="42"/>
+      <c r="N3" s="43"/>
+      <c r="P3" s="38" t="s">
         <v>21</v>
       </c>
-      <c r="Q3" s="34"/>
-      <c r="R3" s="34"/>
-      <c r="S3" s="34"/>
-      <c r="T3" s="34"/>
-      <c r="U3" s="35"/>
-      <c r="V3" s="31" t="s">
+      <c r="Q3" s="39"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="39"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="40"/>
+      <c r="V3" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="W3" s="32"/>
-      <c r="X3" s="32"/>
+      <c r="W3" s="37"/>
+      <c r="X3" s="37"/>
     </row>
     <row r="4" spans="1:24" ht="26" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
@@ -1556,1058 +1416,950 @@
       <c r="X5" s="28"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="31">
         <v>2043</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="31">
         <v>2856</v>
       </c>
-      <c r="F6" s="1">
+      <c r="F6" s="31">
         <v>110453</v>
       </c>
-      <c r="G6" s="6">
+      <c r="G6" s="32">
         <v>45600</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="32">
         <v>45600</v>
       </c>
-      <c r="I6" s="20">
+      <c r="I6" s="33">
         <v>0.99450000000000005</v>
       </c>
-      <c r="J6" s="21">
+      <c r="J6" s="33">
         <v>1</v>
       </c>
-      <c r="K6" s="9">
-        <v>16</v>
-      </c>
-      <c r="L6" s="22">
-        <v>45</v>
-      </c>
-      <c r="M6" s="22">
+      <c r="K6" s="31">
+        <v>17</v>
+      </c>
+      <c r="L6" s="31">
+        <v>46</v>
+      </c>
+      <c r="M6" s="31">
         <v>4</v>
       </c>
-      <c r="N6" s="22">
-        <v>49</v>
-      </c>
-      <c r="O6" s="22">
+      <c r="N6" s="31">
+        <v>50</v>
+      </c>
+      <c r="O6" s="31">
         <v>0</v>
       </c>
-      <c r="P6" s="23"/>
-      <c r="Q6" s="24"/>
-      <c r="R6" s="23"/>
-      <c r="S6" s="27"/>
-      <c r="T6" s="27"/>
-      <c r="U6" s="27"/>
-      <c r="V6" s="1">
+      <c r="P6" s="34"/>
+      <c r="Q6" s="34"/>
+      <c r="R6" s="34"/>
+      <c r="S6" s="35"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="35"/>
+      <c r="V6" s="31">
         <v>5.5</v>
       </c>
-      <c r="W6" s="1">
+      <c r="W6" s="31">
         <v>1</v>
       </c>
-      <c r="X6" s="1">
+      <c r="X6" s="31">
         <v>5.5</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="31">
         <v>2043</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="31">
         <v>2692</v>
       </c>
-      <c r="F7" s="1">
+      <c r="F7" s="31">
         <v>111056</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="32">
         <v>45639</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="32">
         <v>45639</v>
       </c>
-      <c r="I7" s="20">
+      <c r="I7" s="33">
         <v>0.95179999999999998</v>
       </c>
-      <c r="J7" s="21">
-        <v>0.38329999999999997</v>
-      </c>
-      <c r="K7" s="9">
-        <v>15</v>
-      </c>
-      <c r="L7" s="22">
+      <c r="J7" s="33">
+        <v>0.32640000000000002</v>
+      </c>
+      <c r="K7" s="31">
+        <v>16</v>
+      </c>
+      <c r="L7" s="31">
         <v>17</v>
       </c>
-      <c r="M7" s="22">
-        <v>7</v>
-      </c>
-      <c r="N7" s="22">
-        <v>24</v>
-      </c>
-      <c r="O7" s="22">
+      <c r="M7" s="31">
+        <v>7.5</v>
+      </c>
+      <c r="N7" s="31">
+        <v>24.5</v>
+      </c>
+      <c r="O7" s="31">
         <v>1</v>
       </c>
-      <c r="P7" s="23"/>
-      <c r="Q7" s="24"/>
-      <c r="R7" s="23"/>
-      <c r="S7" s="27"/>
-      <c r="T7" s="27"/>
-      <c r="U7" s="27"/>
-      <c r="V7" s="1">
+      <c r="P7" s="34"/>
+      <c r="Q7" s="34"/>
+      <c r="R7" s="34"/>
+      <c r="S7" s="35"/>
+      <c r="T7" s="35"/>
+      <c r="U7" s="35"/>
+      <c r="V7" s="31">
         <v>8</v>
       </c>
-      <c r="W7" s="1">
+      <c r="W7" s="31">
         <v>0.5</v>
       </c>
-      <c r="X7" s="1">
+      <c r="X7" s="31">
         <v>3.5</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="31">
         <v>2043</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="31">
         <v>2692</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="31">
         <v>110575</v>
       </c>
-      <c r="G8" s="6">
+      <c r="G8" s="32">
         <v>45583</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="32">
         <v>45583</v>
       </c>
-      <c r="I8" s="20">
+      <c r="I8" s="33">
         <v>0.88300000000000001</v>
       </c>
-      <c r="J8" s="21">
+      <c r="J8" s="33">
         <v>0.26390000000000002</v>
       </c>
-      <c r="K8" s="9">
-        <v>17</v>
-      </c>
-      <c r="L8" s="22">
+      <c r="K8" s="31">
+        <v>18</v>
+      </c>
+      <c r="L8" s="31">
         <v>20</v>
       </c>
-      <c r="M8" s="22">
+      <c r="M8" s="31">
         <v>1.5</v>
       </c>
-      <c r="N8" s="22">
+      <c r="N8" s="31">
         <v>21.5</v>
       </c>
-      <c r="O8" s="22">
+      <c r="O8" s="31">
         <v>2.5</v>
       </c>
-      <c r="P8" s="23"/>
-      <c r="Q8" s="24"/>
-      <c r="R8" s="23"/>
-      <c r="S8" s="27"/>
-      <c r="T8" s="27"/>
-      <c r="U8" s="27"/>
-      <c r="V8" s="1">
+      <c r="P8" s="34"/>
+      <c r="Q8" s="34"/>
+      <c r="R8" s="34"/>
+      <c r="S8" s="35"/>
+      <c r="T8" s="35"/>
+      <c r="U8" s="35"/>
+      <c r="V8" s="31">
         <v>7</v>
       </c>
-      <c r="W8" s="1">
+      <c r="W8" s="31">
         <v>0.5</v>
       </c>
-      <c r="X8" s="1">
+      <c r="X8" s="31">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="31">
         <v>2043</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="31">
         <v>2043</v>
       </c>
-      <c r="F9" s="1">
-        <v>110105</v>
-      </c>
-      <c r="G9" s="6">
-        <v>45560</v>
-      </c>
-      <c r="H9" s="6">
-        <v>45560</v>
-      </c>
-      <c r="I9" s="20">
-        <v>0.9002</v>
-      </c>
-      <c r="J9" s="21">
-        <v>0.19439999999999999</v>
-      </c>
-      <c r="K9" s="9">
+      <c r="F9" s="31">
+        <v>109998</v>
+      </c>
+      <c r="G9" s="32">
+        <v>45596</v>
+      </c>
+      <c r="H9" s="32">
+        <v>45596</v>
+      </c>
+      <c r="I9" s="33">
+        <v>1</v>
+      </c>
+      <c r="J9" s="33">
+        <v>1</v>
+      </c>
+      <c r="K9" s="31">
         <v>18</v>
       </c>
-      <c r="L9" s="22">
-        <v>16</v>
-      </c>
-      <c r="M9" s="22">
-        <v>3.5</v>
-      </c>
-      <c r="N9" s="22">
+      <c r="L9" s="31">
+        <v>19</v>
+      </c>
+      <c r="M9" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="N9" s="31">
         <v>19.5</v>
       </c>
-      <c r="O9" s="22">
-        <v>5.5</v>
-      </c>
-      <c r="P9" s="23"/>
-      <c r="Q9" s="24"/>
-      <c r="R9" s="23"/>
-      <c r="S9" s="27"/>
-      <c r="T9" s="27"/>
-      <c r="U9" s="27"/>
-      <c r="V9" s="1">
-        <v>6</v>
-      </c>
-      <c r="W9" s="1">
-        <v>2.5</v>
-      </c>
-      <c r="X9" s="1">
-        <v>3</v>
+      <c r="O9" s="31">
+        <v>0</v>
+      </c>
+      <c r="P9" s="34"/>
+      <c r="Q9" s="34"/>
+      <c r="R9" s="34"/>
+      <c r="S9" s="35"/>
+      <c r="T9" s="35"/>
+      <c r="U9" s="35"/>
+      <c r="V9" s="31">
+        <v>5</v>
+      </c>
+      <c r="W9" s="31">
+        <v>2</v>
+      </c>
+      <c r="X9" s="31">
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="31">
         <v>2043</v>
       </c>
-      <c r="E10" s="1">
-        <v>2043</v>
-      </c>
-      <c r="F10" s="1">
-        <v>109998</v>
-      </c>
-      <c r="G10" s="6">
-        <v>45596</v>
-      </c>
-      <c r="H10" s="6">
-        <v>45596</v>
-      </c>
-      <c r="I10" s="20">
+      <c r="E10" s="31">
+        <v>2856</v>
+      </c>
+      <c r="F10" s="31">
+        <v>115047</v>
+      </c>
+      <c r="G10" s="32">
+        <v>45944</v>
+      </c>
+      <c r="H10" s="32">
+        <v>45944</v>
+      </c>
+      <c r="I10" s="33">
+        <v>0.755</v>
+      </c>
+      <c r="J10" s="33">
         <v>1</v>
       </c>
-      <c r="J10" s="21">
-        <v>1</v>
-      </c>
-      <c r="K10" s="9">
-        <v>17</v>
-      </c>
-      <c r="L10" s="22">
-        <v>19</v>
-      </c>
-      <c r="M10" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N10" s="22">
-        <v>19.5</v>
-      </c>
-      <c r="O10" s="22">
+      <c r="K10" s="31">
+        <v>6</v>
+      </c>
+      <c r="L10" s="31">
+        <v>12</v>
+      </c>
+      <c r="M10" s="31">
+        <v>1.5</v>
+      </c>
+      <c r="N10" s="31">
+        <v>13.5</v>
+      </c>
+      <c r="O10" s="31">
         <v>0</v>
       </c>
-      <c r="P10" s="23"/>
-      <c r="Q10" s="24"/>
-      <c r="R10" s="23"/>
-      <c r="S10" s="27"/>
-      <c r="T10" s="27"/>
-      <c r="U10" s="27"/>
-      <c r="V10" s="1">
-        <v>5</v>
-      </c>
-      <c r="W10" s="1">
+      <c r="P10" s="34"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="35"/>
+      <c r="T10" s="35"/>
+      <c r="U10" s="35"/>
+      <c r="V10" s="31">
+        <v>8.5</v>
+      </c>
+      <c r="W10" s="31">
         <v>2</v>
       </c>
-      <c r="X10" s="1">
-        <v>2</v>
+      <c r="X10" s="31">
+        <v>1.5</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="31">
         <v>2043</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="31">
         <v>2856</v>
       </c>
-      <c r="F11" s="1">
-        <v>109819</v>
-      </c>
-      <c r="G11" s="6">
-        <v>45562</v>
-      </c>
-      <c r="H11" s="6">
-        <v>45562</v>
-      </c>
-      <c r="I11" s="20">
-        <v>0.9224</v>
-      </c>
-      <c r="J11" s="21">
-        <v>0.1875</v>
-      </c>
-      <c r="K11" s="9">
-        <v>18</v>
-      </c>
-      <c r="L11" s="22">
-        <v>16</v>
-      </c>
-      <c r="M11" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="N11" s="22">
-        <v>18.5</v>
-      </c>
-      <c r="O11" s="22">
-        <v>5</v>
-      </c>
-      <c r="P11" s="23"/>
-      <c r="Q11" s="24"/>
-      <c r="R11" s="23"/>
-      <c r="S11" s="27"/>
-      <c r="T11" s="27"/>
-      <c r="U11" s="27"/>
-      <c r="V11" s="1">
-        <v>7.5</v>
-      </c>
-      <c r="W11" s="1">
+      <c r="F11" s="31">
+        <v>114100</v>
+      </c>
+      <c r="G11" s="32">
+        <v>45863</v>
+      </c>
+      <c r="H11" s="32">
+        <v>45863</v>
+      </c>
+      <c r="I11" s="33">
+        <v>0.755</v>
+      </c>
+      <c r="J11" s="33">
+        <v>0.34720000000000001</v>
+      </c>
+      <c r="K11" s="31">
+        <v>9</v>
+      </c>
+      <c r="L11" s="31">
+        <v>13</v>
+      </c>
+      <c r="M11" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="N11" s="31">
+        <v>13.5</v>
+      </c>
+      <c r="O11" s="31">
+        <v>1</v>
+      </c>
+      <c r="P11" s="34"/>
+      <c r="Q11" s="34"/>
+      <c r="R11" s="34"/>
+      <c r="S11" s="35"/>
+      <c r="T11" s="35"/>
+      <c r="U11" s="35"/>
+      <c r="V11" s="31">
+        <v>5.5</v>
+      </c>
+      <c r="W11" s="31">
+        <v>1</v>
+      </c>
+      <c r="X11" s="31">
         <v>2</v>
-      </c>
-      <c r="X11" s="1">
-        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="31">
         <v>2043</v>
       </c>
-      <c r="E12" s="1">
-        <v>2856</v>
-      </c>
-      <c r="F12" s="1">
-        <v>115047</v>
-      </c>
-      <c r="G12" s="6">
-        <v>45944</v>
-      </c>
-      <c r="H12" s="6">
-        <v>45944</v>
-      </c>
-      <c r="I12" s="20">
+      <c r="E12" s="31">
+        <v>2043</v>
+      </c>
+      <c r="F12" s="31">
+        <v>115404</v>
+      </c>
+      <c r="G12" s="32">
+        <v>45986</v>
+      </c>
+      <c r="H12" s="32">
+        <v>45986</v>
+      </c>
+      <c r="I12" s="33">
         <v>0.755</v>
       </c>
-      <c r="J12" s="21">
+      <c r="J12" s="33">
         <v>1</v>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="31">
         <v>5</v>
       </c>
-      <c r="L12" s="22">
-        <v>12</v>
-      </c>
-      <c r="M12" s="22">
-        <v>1.5</v>
-      </c>
-      <c r="N12" s="22">
-        <v>13.5</v>
-      </c>
-      <c r="O12" s="22">
+      <c r="L12" s="31">
+        <v>9</v>
+      </c>
+      <c r="M12" s="31">
+        <v>2.5</v>
+      </c>
+      <c r="N12" s="31">
+        <v>11.5</v>
+      </c>
+      <c r="O12" s="31">
         <v>0</v>
       </c>
-      <c r="P12" s="23"/>
-      <c r="Q12" s="24"/>
-      <c r="R12" s="23"/>
-      <c r="S12" s="27"/>
-      <c r="T12" s="27"/>
-      <c r="U12" s="27"/>
-      <c r="V12" s="1">
-        <v>8.5</v>
-      </c>
-      <c r="W12" s="1">
-        <v>2</v>
-      </c>
-      <c r="X12" s="1">
-        <v>1.5</v>
+      <c r="P12" s="34"/>
+      <c r="Q12" s="34"/>
+      <c r="R12" s="34"/>
+      <c r="S12" s="35"/>
+      <c r="T12" s="35"/>
+      <c r="U12" s="35"/>
+      <c r="V12" s="31">
+        <v>8</v>
+      </c>
+      <c r="W12" s="31">
+        <v>1</v>
+      </c>
+      <c r="X12" s="31">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="31">
         <v>2043</v>
       </c>
-      <c r="E13" s="1">
-        <v>2856</v>
-      </c>
-      <c r="F13" s="1">
-        <v>114100</v>
-      </c>
-      <c r="G13" s="6">
-        <v>45863</v>
-      </c>
-      <c r="H13" s="6">
-        <v>45863</v>
-      </c>
-      <c r="I13" s="20">
+      <c r="E13" s="31">
+        <v>2692</v>
+      </c>
+      <c r="F13" s="31">
+        <v>113450</v>
+      </c>
+      <c r="G13" s="32">
+        <v>45852</v>
+      </c>
+      <c r="H13" s="32">
+        <v>45852</v>
+      </c>
+      <c r="I13" s="33">
         <v>0.755</v>
       </c>
-      <c r="J13" s="21">
-        <v>0.34720000000000001</v>
-      </c>
-      <c r="K13" s="9">
-        <v>8</v>
-      </c>
-      <c r="L13" s="22">
-        <v>13</v>
-      </c>
-      <c r="M13" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N13" s="22">
-        <v>13.5</v>
-      </c>
-      <c r="O13" s="22">
+      <c r="J13" s="33">
+        <v>0.29170000000000001</v>
+      </c>
+      <c r="K13" s="31">
+        <v>9</v>
+      </c>
+      <c r="L13" s="31">
+        <v>9</v>
+      </c>
+      <c r="M13" s="31">
+        <v>2.5</v>
+      </c>
+      <c r="N13" s="31">
+        <v>11.5</v>
+      </c>
+      <c r="O13" s="31">
         <v>1</v>
       </c>
-      <c r="P13" s="23"/>
-      <c r="Q13" s="24"/>
-      <c r="R13" s="23"/>
-      <c r="S13" s="27"/>
-      <c r="T13" s="27"/>
-      <c r="U13" s="27"/>
-      <c r="V13" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="W13" s="1">
+      <c r="P13" s="34"/>
+      <c r="Q13" s="34"/>
+      <c r="R13" s="34"/>
+      <c r="S13" s="35"/>
+      <c r="T13" s="35"/>
+      <c r="U13" s="35"/>
+      <c r="V13" s="31">
+        <v>7</v>
+      </c>
+      <c r="W13" s="31">
+        <v>2</v>
+      </c>
+      <c r="X13" s="31">
         <v>1</v>
-      </c>
-      <c r="X13" s="1">
-        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="31">
         <v>2043</v>
       </c>
-      <c r="E14" s="1">
-        <v>2043</v>
-      </c>
-      <c r="F14" s="1">
-        <v>115404</v>
-      </c>
-      <c r="G14" s="6">
-        <v>45986</v>
-      </c>
-      <c r="H14" s="6">
-        <v>45986</v>
-      </c>
-      <c r="I14" s="20">
-        <v>0.755</v>
-      </c>
-      <c r="J14" s="21">
-        <v>1</v>
-      </c>
-      <c r="K14" s="9">
-        <v>4</v>
-      </c>
-      <c r="L14" s="22">
-        <v>9</v>
-      </c>
-      <c r="M14" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="N14" s="22">
+      <c r="E14" s="31">
+        <v>2856</v>
+      </c>
+      <c r="F14" s="31">
+        <v>111960</v>
+      </c>
+      <c r="G14" s="32">
+        <v>45707</v>
+      </c>
+      <c r="H14" s="32">
+        <v>45707</v>
+      </c>
+      <c r="I14" s="33">
+        <v>0.78500000000000003</v>
+      </c>
+      <c r="J14" s="33">
+        <v>0.1583</v>
+      </c>
+      <c r="K14" s="31">
+        <v>14</v>
+      </c>
+      <c r="L14" s="31">
+        <v>11</v>
+      </c>
+      <c r="M14" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="N14" s="31">
         <v>11.5</v>
       </c>
-      <c r="O14" s="22">
-        <v>0</v>
-      </c>
-      <c r="P14" s="23"/>
-      <c r="Q14" s="24"/>
-      <c r="R14" s="23"/>
-      <c r="S14" s="27"/>
-      <c r="T14" s="27"/>
-      <c r="U14" s="27"/>
-      <c r="V14" s="1">
-        <v>8</v>
-      </c>
-      <c r="W14" s="1">
-        <v>1</v>
-      </c>
-      <c r="X14" s="1">
+      <c r="O14" s="31">
+        <v>2</v>
+      </c>
+      <c r="P14" s="34"/>
+      <c r="Q14" s="34"/>
+      <c r="R14" s="34"/>
+      <c r="S14" s="35"/>
+      <c r="T14" s="35"/>
+      <c r="U14" s="35"/>
+      <c r="V14" s="31">
+        <v>6</v>
+      </c>
+      <c r="W14" s="31">
+        <v>3</v>
+      </c>
+      <c r="X14" s="31">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="31">
         <v>2043</v>
       </c>
-      <c r="E15" s="1">
-        <v>2692</v>
-      </c>
-      <c r="F15" s="1">
-        <v>113450</v>
-      </c>
-      <c r="G15" s="6">
-        <v>45852</v>
-      </c>
-      <c r="H15" s="6">
-        <v>45852</v>
-      </c>
-      <c r="I15" s="20">
+      <c r="E15" s="31">
+        <v>2043</v>
+      </c>
+      <c r="F15" s="31">
+        <v>113076</v>
+      </c>
+      <c r="G15" s="32">
+        <v>45806</v>
+      </c>
+      <c r="H15" s="32">
+        <v>45806</v>
+      </c>
+      <c r="I15" s="33">
         <v>0.755</v>
       </c>
-      <c r="J15" s="21">
-        <v>0.29170000000000001</v>
-      </c>
-      <c r="K15" s="9">
-        <v>8</v>
-      </c>
-      <c r="L15" s="22">
-        <v>9</v>
-      </c>
-      <c r="M15" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="N15" s="22">
-        <v>11.5</v>
-      </c>
-      <c r="O15" s="22">
+      <c r="J15" s="33">
         <v>1</v>
       </c>
-      <c r="P15" s="23"/>
-      <c r="Q15" s="24"/>
-      <c r="R15" s="23"/>
-      <c r="S15" s="27"/>
-      <c r="T15" s="27"/>
-      <c r="U15" s="27"/>
-      <c r="V15" s="1">
+      <c r="K15" s="31">
+        <v>11</v>
+      </c>
+      <c r="L15" s="31">
         <v>7</v>
       </c>
-      <c r="W15" s="1">
+      <c r="M15" s="31">
+        <v>3.5</v>
+      </c>
+      <c r="N15" s="31">
+        <v>10.5</v>
+      </c>
+      <c r="O15" s="31">
+        <v>0</v>
+      </c>
+      <c r="P15" s="34"/>
+      <c r="Q15" s="34"/>
+      <c r="R15" s="34"/>
+      <c r="S15" s="35"/>
+      <c r="T15" s="35"/>
+      <c r="U15" s="35"/>
+      <c r="V15" s="31">
+        <v>5.5</v>
+      </c>
+      <c r="W15" s="31">
         <v>2</v>
       </c>
-      <c r="X15" s="1">
-        <v>1</v>
+      <c r="X15" s="31">
+        <v>1.5</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="31">
         <v>2043</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="31">
         <v>2856</v>
       </c>
-      <c r="F16" s="1">
-        <v>111960</v>
-      </c>
-      <c r="G16" s="6">
-        <v>45707</v>
-      </c>
-      <c r="H16" s="6">
-        <v>45707</v>
-      </c>
-      <c r="I16" s="20">
-        <v>0.78500000000000003</v>
-      </c>
-      <c r="J16" s="21">
-        <v>0.1583</v>
-      </c>
-      <c r="K16" s="9">
-        <v>13</v>
-      </c>
-      <c r="L16" s="22">
-        <v>11</v>
-      </c>
-      <c r="M16" s="22">
+      <c r="F16" s="31">
+        <v>116060</v>
+      </c>
+      <c r="G16" s="32">
+        <v>46010</v>
+      </c>
+      <c r="H16" s="32">
+        <v>46010</v>
+      </c>
+      <c r="I16" s="33">
+        <v>0.755</v>
+      </c>
+      <c r="J16" s="33">
+        <v>1</v>
+      </c>
+      <c r="K16" s="31">
+        <v>4</v>
+      </c>
+      <c r="L16" s="31">
+        <v>8</v>
+      </c>
+      <c r="M16" s="31">
         <v>0.5</v>
       </c>
-      <c r="N16" s="22">
-        <v>11.5</v>
-      </c>
-      <c r="O16" s="22">
-        <v>2</v>
-      </c>
-      <c r="P16" s="23"/>
-      <c r="Q16" s="24"/>
-      <c r="R16" s="23"/>
-      <c r="S16" s="27"/>
-      <c r="T16" s="27"/>
-      <c r="U16" s="27"/>
-      <c r="V16" s="1">
+      <c r="N16" s="31">
+        <v>8.5</v>
+      </c>
+      <c r="O16" s="31">
+        <v>0</v>
+      </c>
+      <c r="P16" s="34"/>
+      <c r="Q16" s="34"/>
+      <c r="R16" s="34"/>
+      <c r="S16" s="35"/>
+      <c r="T16" s="35"/>
+      <c r="U16" s="35"/>
+      <c r="V16" s="31">
         <v>6</v>
       </c>
-      <c r="W16" s="1">
-        <v>3</v>
-      </c>
-      <c r="X16" s="1">
-        <v>0</v>
+      <c r="W16" s="31">
+        <v>1</v>
+      </c>
+      <c r="X16" s="31">
+        <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="31">
         <v>2043</v>
       </c>
-      <c r="E17" s="1">
-        <v>2043</v>
-      </c>
-      <c r="F17" s="1">
-        <v>113076</v>
-      </c>
-      <c r="G17" s="6">
-        <v>45806</v>
-      </c>
-      <c r="H17" s="6">
-        <v>45806</v>
-      </c>
-      <c r="I17" s="20">
+      <c r="E17" s="31">
+        <v>2692</v>
+      </c>
+      <c r="F17" s="31">
+        <v>114157</v>
+      </c>
+      <c r="G17" s="32">
+        <v>45904</v>
+      </c>
+      <c r="H17" s="32">
+        <v>45904</v>
+      </c>
+      <c r="I17" s="33">
         <v>0.755</v>
       </c>
-      <c r="J17" s="21">
+      <c r="J17" s="33">
+        <v>0.19439999999999999</v>
+      </c>
+      <c r="K17" s="31">
+        <v>7</v>
+      </c>
+      <c r="L17" s="31">
+        <v>7</v>
+      </c>
+      <c r="M17" s="31">
         <v>1</v>
       </c>
-      <c r="K17" s="9">
-        <v>10</v>
-      </c>
-      <c r="L17" s="22">
-        <v>7</v>
-      </c>
-      <c r="M17" s="22">
-        <v>3.5</v>
-      </c>
-      <c r="N17" s="22">
-        <v>10.5</v>
-      </c>
-      <c r="O17" s="22">
+      <c r="N17" s="31">
+        <v>8</v>
+      </c>
+      <c r="O17" s="31">
+        <v>1</v>
+      </c>
+      <c r="P17" s="34"/>
+      <c r="Q17" s="34"/>
+      <c r="R17" s="34"/>
+      <c r="S17" s="35"/>
+      <c r="T17" s="35"/>
+      <c r="U17" s="35"/>
+      <c r="V17" s="31">
+        <v>6</v>
+      </c>
+      <c r="W17" s="31">
         <v>0</v>
       </c>
-      <c r="P17" s="23"/>
-      <c r="Q17" s="24"/>
-      <c r="R17" s="23"/>
-      <c r="S17" s="27"/>
-      <c r="T17" s="27"/>
-      <c r="U17" s="27"/>
-      <c r="V17" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="W17" s="1">
-        <v>2</v>
-      </c>
-      <c r="X17" s="1">
-        <v>1.5</v>
+      <c r="X17" s="31">
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="31">
         <v>2043</v>
       </c>
-      <c r="E18" s="1">
-        <v>2043</v>
-      </c>
-      <c r="F18" s="1">
-        <v>112083</v>
-      </c>
-      <c r="G18" s="6">
-        <v>45736</v>
-      </c>
-      <c r="H18" s="6">
-        <v>45736</v>
-      </c>
-      <c r="I18" s="20">
+      <c r="E18" s="31">
+        <v>2692</v>
+      </c>
+      <c r="F18" s="31">
+        <v>114431</v>
+      </c>
+      <c r="G18" s="32">
+        <v>45930</v>
+      </c>
+      <c r="H18" s="32">
+        <v>45930</v>
+      </c>
+      <c r="I18" s="33">
         <v>0.755</v>
       </c>
-      <c r="J18" s="21">
+      <c r="J18" s="33">
         <v>1</v>
       </c>
-      <c r="K18" s="9">
-        <v>12</v>
-      </c>
-      <c r="L18" s="22">
+      <c r="K18" s="31">
+        <v>7</v>
+      </c>
+      <c r="L18" s="31">
         <v>6</v>
       </c>
-      <c r="M18" s="22">
-        <v>3</v>
-      </c>
-      <c r="N18" s="22">
-        <v>9</v>
-      </c>
-      <c r="O18" s="22">
+      <c r="M18" s="31">
+        <v>0.5</v>
+      </c>
+      <c r="N18" s="31">
+        <v>6.5</v>
+      </c>
+      <c r="O18" s="31">
         <v>0</v>
       </c>
-      <c r="P18" s="23"/>
-      <c r="Q18" s="24"/>
-      <c r="R18" s="23"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
-      <c r="U18" s="27"/>
-      <c r="V18" s="1">
-        <v>5.5</v>
-      </c>
-      <c r="W18" s="1">
+      <c r="P18" s="34"/>
+      <c r="Q18" s="34"/>
+      <c r="R18" s="34"/>
+      <c r="S18" s="35"/>
+      <c r="T18" s="35"/>
+      <c r="U18" s="35"/>
+      <c r="V18" s="31">
+        <v>4.5</v>
+      </c>
+      <c r="W18" s="31">
+        <v>2</v>
+      </c>
+      <c r="X18" s="31">
         <v>0</v>
-      </c>
-      <c r="X18" s="1">
-        <v>1.5</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="31">
         <v>2043</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="31">
         <v>2856</v>
       </c>
-      <c r="F19" s="1">
-        <v>116060</v>
-      </c>
-      <c r="G19" s="6">
-        <v>46010</v>
-      </c>
-      <c r="H19" s="6">
-        <v>46010</v>
-      </c>
-      <c r="I19" s="20">
+      <c r="F19" s="31">
+        <v>112522</v>
+      </c>
+      <c r="G19" s="32">
+        <v>45776</v>
+      </c>
+      <c r="H19" s="32">
+        <v>45776</v>
+      </c>
+      <c r="I19" s="33">
         <v>0.755</v>
       </c>
-      <c r="J19" s="21">
+      <c r="J19" s="33">
         <v>1</v>
       </c>
-      <c r="K19" s="9">
-        <v>3</v>
-      </c>
-      <c r="L19" s="22">
-        <v>8</v>
-      </c>
-      <c r="M19" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N19" s="22">
-        <v>8.5</v>
-      </c>
-      <c r="O19" s="22">
+      <c r="K19" s="31">
+        <v>12</v>
+      </c>
+      <c r="L19" s="31">
+        <v>6</v>
+      </c>
+      <c r="M19" s="31">
         <v>0</v>
       </c>
-      <c r="P19" s="23"/>
-      <c r="Q19" s="24"/>
-      <c r="R19" s="23"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="27"/>
-      <c r="V19" s="1">
+      <c r="N19" s="31">
         <v>6</v>
       </c>
-      <c r="W19" s="1">
-        <v>1</v>
-      </c>
-      <c r="X19" s="1">
-        <v>1.5</v>
+      <c r="O19" s="31">
+        <v>0</v>
+      </c>
+      <c r="P19" s="34"/>
+      <c r="Q19" s="34"/>
+      <c r="R19" s="34"/>
+      <c r="S19" s="35"/>
+      <c r="T19" s="35"/>
+      <c r="U19" s="35"/>
+      <c r="V19" s="31">
+        <v>4</v>
+      </c>
+      <c r="W19" s="31">
+        <v>0</v>
+      </c>
+      <c r="X19" s="31">
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="1">
-        <v>2043</v>
-      </c>
-      <c r="E20" s="1">
-        <v>2692</v>
-      </c>
-      <c r="F20" s="1">
-        <v>114157</v>
-      </c>
-      <c r="G20" s="6">
-        <v>45904</v>
-      </c>
-      <c r="H20" s="6">
-        <v>45904</v>
-      </c>
-      <c r="I20" s="20">
-        <v>0.755</v>
-      </c>
-      <c r="J20" s="21">
-        <v>0.29170000000000001</v>
-      </c>
-      <c r="K20" s="9">
-        <v>6</v>
-      </c>
-      <c r="L20" s="22">
-        <v>7</v>
-      </c>
-      <c r="M20" s="22">
-        <v>1</v>
-      </c>
-      <c r="N20" s="22">
-        <v>8</v>
-      </c>
-      <c r="O20" s="22">
-        <v>1</v>
-      </c>
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="20"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="22"/>
+      <c r="M20" s="22"/>
+      <c r="N20" s="22"/>
+      <c r="O20" s="22"/>
       <c r="P20" s="23"/>
       <c r="Q20" s="24"/>
       <c r="R20" s="23"/>
       <c r="S20" s="27"/>
       <c r="T20" s="27"/>
       <c r="U20" s="27"/>
-      <c r="V20" s="1">
-        <v>6</v>
-      </c>
-      <c r="W20" s="1">
-        <v>0</v>
-      </c>
-      <c r="X20" s="1">
-        <v>1</v>
-      </c>
+      <c r="V20" s="1"/>
+      <c r="W20" s="1"/>
+      <c r="X20" s="1"/>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="1">
-        <v>2043</v>
-      </c>
-      <c r="E21" s="1">
-        <v>2692</v>
-      </c>
-      <c r="F21" s="1">
-        <v>114431</v>
-      </c>
-      <c r="G21" s="6">
-        <v>45930</v>
-      </c>
-      <c r="H21" s="6">
-        <v>45930</v>
-      </c>
-      <c r="I21" s="20">
-        <v>0.755</v>
-      </c>
-      <c r="J21" s="21">
-        <v>1</v>
-      </c>
-      <c r="K21" s="9">
-        <v>6</v>
-      </c>
-      <c r="L21" s="22">
-        <v>6</v>
-      </c>
-      <c r="M21" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N21" s="22">
-        <v>6.5</v>
-      </c>
-      <c r="O21" s="22">
-        <v>0</v>
-      </c>
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="22"/>
       <c r="P21" s="23"/>
       <c r="Q21" s="24"/>
       <c r="R21" s="23"/>
       <c r="S21" s="27"/>
       <c r="T21" s="27"/>
       <c r="U21" s="27"/>
-      <c r="V21" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="W21" s="1">
-        <v>2</v>
-      </c>
-      <c r="X21" s="1">
-        <v>0</v>
-      </c>
+      <c r="V21" s="1"/>
+      <c r="W21" s="1"/>
+      <c r="X21" s="1"/>
     </row>
     <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A22" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D22" s="1">
-        <v>2043</v>
-      </c>
-      <c r="E22" s="1">
-        <v>2856</v>
-      </c>
-      <c r="F22" s="1">
-        <v>112522</v>
-      </c>
-      <c r="G22" s="6">
-        <v>45776</v>
-      </c>
-      <c r="H22" s="6">
-        <v>45776</v>
-      </c>
-      <c r="I22" s="20">
-        <v>0.755</v>
-      </c>
-      <c r="J22" s="21">
-        <v>1</v>
-      </c>
-      <c r="K22" s="9">
-        <v>11</v>
-      </c>
-      <c r="L22" s="22">
-        <v>6</v>
-      </c>
-      <c r="M22" s="22">
-        <v>0</v>
-      </c>
-      <c r="N22" s="22">
-        <v>6</v>
-      </c>
-      <c r="O22" s="22">
-        <v>0</v>
-      </c>
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="22"/>
+      <c r="N22" s="22"/>
+      <c r="O22" s="22"/>
       <c r="P22" s="23"/>
       <c r="Q22" s="24"/>
       <c r="R22" s="23"/>
       <c r="S22" s="27"/>
       <c r="T22" s="27"/>
       <c r="U22" s="27"/>
-      <c r="V22" s="1">
-        <v>4</v>
-      </c>
-      <c r="W22" s="1">
-        <v>0</v>
-      </c>
-      <c r="X22" s="1">
-        <v>2</v>
-      </c>
+      <c r="V22" s="1"/>
+      <c r="W22" s="1"/>
+      <c r="X22" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2615,44 +2367,44 @@
     <mergeCell ref="P3:U3"/>
     <mergeCell ref="L3:N3"/>
   </mergeCells>
-  <conditionalFormatting sqref="A22:K22 U6:U22 A6:K21">
+  <conditionalFormatting sqref="A20:K22 U20:U22">
     <cfRule type="expression" dxfId="6" priority="8" stopIfTrue="1">
-      <formula>$B6&lt;&gt;""</formula>
+      <formula>$B20&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I22">
+  <conditionalFormatting sqref="I20:I22">
     <cfRule type="expression" dxfId="5" priority="7" stopIfTrue="1">
-      <formula>AND($B6&lt;&gt;"",$L6&lt;0.85)</formula>
+      <formula>AND($B20&lt;&gt;"",$L20&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J6:J22">
+  <conditionalFormatting sqref="J20:J22">
     <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
-      <formula>AND($B6&lt;&gt;"",$M$29&lt;0.85)</formula>
+      <formula>AND($B20&lt;&gt;"",$M$29&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L6:T22">
+  <conditionalFormatting sqref="L20:T22">
     <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
-      <formula>$B6&lt;&gt;""</formula>
+      <formula>$B20&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:V22">
+  <conditionalFormatting sqref="V20:V22">
     <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
-      <formula>AND($B6&lt;&gt;"",$Z6&lt;1)</formula>
+      <formula>AND($B20&lt;&gt;"",$Z20&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:X22">
+  <conditionalFormatting sqref="V20:X22">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
-      <formula>$B6&lt;&gt;""</formula>
+      <formula>$B20&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W6:W22">
+  <conditionalFormatting sqref="W20:W22">
     <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
-      <formula>AND($B6&lt;&gt;"",$AA6&lt;1)</formula>
+      <formula>AND($B20&lt;&gt;"",$AA20&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X6:X22">
+  <conditionalFormatting sqref="X20:X22">
     <cfRule type="expression" priority="3" stopIfTrue="1">
-      <formula>AND($B6&lt;&gt;"",$AB6&lt;1)</formula>
+      <formula>AND($B20&lt;&gt;"",$AB20&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-20 12:19)
</commit_message>
<xml_diff>
--- a/camino_cumbre/CAMINO A LA CUMBRE.xlsx
+++ b/camino_cumbre/CAMINO A LA CUMBRE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/camino_cumbre/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94494843-618C-B24C-890B-7D94748204C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9E17CE6-A9C4-154A-9F92-E62EE77455D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="1140" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="42">
   <si>
     <t>Dir. de Venta</t>
   </si>
@@ -161,7 +161,7 @@
     <t>Pólizas Pagadas</t>
   </si>
   <si>
-    <t>Avance  al 31 de marzo de 2026.</t>
+    <t>Avance  al 15 de abril de 2026.</t>
   </si>
 </sst>
 </file>
@@ -501,39 +501,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{5777CE91-9B5C-AD4F-B1FB-47F4B57F6892}"/>
     <cellStyle name="Porcentaje 2" xfId="2" xr:uid="{7B24C14E-EE44-314E-8590-6F0AEF4F900D}"/>
   </cellStyles>
-  <dxfs count="24">
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="28">
     <dxf>
       <font>
         <b/>
@@ -542,6 +510,116 @@
         <extend val="0"/>
         <color indexed="10"/>
       </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -859,8 +937,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X22" totalsRowShown="0" headerRowDxfId="23" headerRowBorderDxfId="22" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
-  <autoFilter ref="A4:X22" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X21" totalsRowShown="0" headerRowDxfId="27" headerRowBorderDxfId="26" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
+  <autoFilter ref="A4:X21" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}"/>
   <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{452BBEC3-C02A-954A-AF30-AAC8D4135219}" name="Dir. de Venta" dataCellStyle="Normal 2"/>
     <tableColumn id="2" xr3:uid="{96963370-19D6-F44C-A2DA-2A40ED43DD5C}" name="Oficina" dataCellStyle="Normal 2"/>
@@ -868,21 +946,21 @@
     <tableColumn id="4" xr3:uid="{E64AD030-9FFA-1B49-B7F8-31458F00EB96}" name="Mat" dataCellStyle="Normal 2"/>
     <tableColumn id="5" xr3:uid="{407858BC-0878-5E44-A050-843285231653}" name="Suc" dataCellStyle="Normal 2"/>
     <tableColumn id="6" xr3:uid="{6FEB1162-A9E3-244F-886A-8D5C735D8BE4}" name="Asesor" dataCellStyle="Normal 2"/>
-    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="21" dataCellStyle="Normal 2"/>
-    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="20" dataCellStyle="Normal 2"/>
-    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="19" dataCellStyle="Porcentaje 2"/>
-    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="18" dataCellStyle="Normal 2"/>
-    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="17" dataCellStyle="Normal 2"/>
-    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="16" dataCellStyle="Normal 2"/>
-    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="15" dataCellStyle="Normal 2"/>
-    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="14" dataCellStyle="Normal 2"/>
-    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="13" dataCellStyle="Normal 2"/>
-    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="12" dataCellStyle="Normal 2"/>
-    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="11" dataCellStyle="Normal 2"/>
-    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="10" dataCellStyle="Normal 2"/>
-    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="9" dataCellStyle="Normal 2"/>
-    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="8" dataCellStyle="Normal 2"/>
-    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="7" dataCellStyle="Normal 2"/>
+    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="25" dataCellStyle="Normal 2"/>
+    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="24" dataCellStyle="Normal 2"/>
+    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="23" dataCellStyle="Porcentaje 2"/>
+    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="22" dataCellStyle="Normal 2"/>
+    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="21" dataCellStyle="Normal 2"/>
+    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="20" dataCellStyle="Normal 2"/>
+    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="19" dataCellStyle="Normal 2"/>
+    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="18" dataCellStyle="Normal 2"/>
+    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="17" dataCellStyle="Normal 2"/>
+    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="16" dataCellStyle="Normal 2"/>
+    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="15" dataCellStyle="Normal 2"/>
+    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="14" dataCellStyle="Normal 2"/>
+    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="13" dataCellStyle="Normal 2"/>
+    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="12" dataCellStyle="Normal 2"/>
+    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="11" dataCellStyle="Normal 2"/>
     <tableColumn id="22" xr3:uid="{FB6CEF72-668C-CB49-ACCA-75A997C036A1}" name="Mes 1" dataCellStyle="Normal 2"/>
     <tableColumn id="23" xr3:uid="{58B1F16B-3FBB-3D4C-8C16-DD05D985324B}" name="Mes 2" dataCellStyle="Normal 2"/>
     <tableColumn id="24" xr3:uid="{B5A4E59E-794B-AB4B-BB2B-840B78865464}" name="Mes 3" dataCellStyle="Normal 2"/>
@@ -1208,7 +1286,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54AB4B63-646E-974E-8074-72018385EA77}">
-  <dimension ref="A1:X22"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
@@ -1369,7 +1447,7 @@
       </c>
       <c r="O5" s="15"/>
       <c r="P5" s="19">
-        <f t="shared" ref="P5:U5" si="0">COUNTIF(P6:P65513,"p")</f>
+        <f t="shared" ref="P5:U5" si="0">COUNTIF(P6:P65512,"p")</f>
         <v>0</v>
       </c>
       <c r="Q5" s="19">
@@ -1428,16 +1506,16 @@
         <v>1</v>
       </c>
       <c r="K6" s="9">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="L6" s="22">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M6" s="22">
         <v>4</v>
       </c>
       <c r="N6" s="22">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O6" s="22">
         <v>0</v>
@@ -1472,7 +1550,7 @@
         <v>2043</v>
       </c>
       <c r="E7" s="1">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="F7" s="1">
         <v>111056</v>
@@ -1490,7 +1568,7 @@
         <v>0.32640000000000002</v>
       </c>
       <c r="K7" s="9">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="L7" s="22">
         <v>17</v>
@@ -1534,37 +1612,37 @@
         <v>2043</v>
       </c>
       <c r="E8" s="1">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="F8" s="1">
-        <v>110575</v>
+        <v>115047</v>
       </c>
       <c r="G8" s="6">
-        <v>45583</v>
+        <v>45944</v>
       </c>
       <c r="H8" s="6">
-        <v>45583</v>
+        <v>45944</v>
       </c>
       <c r="I8" s="20">
-        <v>0.88970000000000005</v>
+        <v>0.755</v>
       </c>
       <c r="J8" s="21">
-        <v>0.26390000000000002</v>
+        <v>1</v>
       </c>
       <c r="K8" s="9">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="L8" s="22">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="M8" s="22">
         <v>1.5</v>
       </c>
       <c r="N8" s="22">
-        <v>21.5</v>
+        <v>14.5</v>
       </c>
       <c r="O8" s="22">
-        <v>2.5</v>
+        <v>0</v>
       </c>
       <c r="P8" s="23"/>
       <c r="Q8" s="24"/>
@@ -1573,13 +1651,13 @@
       <c r="T8" s="27"/>
       <c r="U8" s="27"/>
       <c r="V8" s="1">
-        <v>7</v>
+        <v>8.5</v>
       </c>
       <c r="W8" s="1">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="X8" s="1">
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
@@ -1596,37 +1674,37 @@
         <v>2043</v>
       </c>
       <c r="E9" s="1">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="F9" s="1">
-        <v>109998</v>
+        <v>114100</v>
       </c>
       <c r="G9" s="6">
-        <v>45596</v>
+        <v>45863</v>
       </c>
       <c r="H9" s="6">
-        <v>45596</v>
+        <v>45863</v>
       </c>
       <c r="I9" s="20">
-        <v>1</v>
+        <v>0.755</v>
       </c>
       <c r="J9" s="21">
-        <v>1</v>
+        <v>0.26040000000000002</v>
       </c>
       <c r="K9" s="9">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="L9" s="22">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="M9" s="22">
         <v>0.5</v>
       </c>
       <c r="N9" s="22">
-        <v>19.5</v>
+        <v>13.5</v>
       </c>
       <c r="O9" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P9" s="23"/>
       <c r="Q9" s="24"/>
@@ -1635,10 +1713,10 @@
       <c r="T9" s="27"/>
       <c r="U9" s="27"/>
       <c r="V9" s="1">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="W9" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X9" s="1">
         <v>2</v>
@@ -1658,16 +1736,16 @@
         <v>2043</v>
       </c>
       <c r="E10" s="1">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="F10" s="1">
-        <v>115047</v>
+        <v>115404</v>
       </c>
       <c r="G10" s="6">
-        <v>45944</v>
+        <v>45986</v>
       </c>
       <c r="H10" s="6">
-        <v>45944</v>
+        <v>45986</v>
       </c>
       <c r="I10" s="20">
         <v>0.755</v>
@@ -1679,13 +1757,13 @@
         <v>6</v>
       </c>
       <c r="L10" s="22">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="M10" s="22">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="N10" s="22">
-        <v>14.5</v>
+        <v>12</v>
       </c>
       <c r="O10" s="22">
         <v>0</v>
@@ -1697,13 +1775,13 @@
       <c r="T10" s="27"/>
       <c r="U10" s="27"/>
       <c r="V10" s="1">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="W10" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X10" s="1">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
@@ -1720,34 +1798,34 @@
         <v>2043</v>
       </c>
       <c r="E11" s="1">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="F11" s="1">
-        <v>114100</v>
+        <v>113450</v>
       </c>
       <c r="G11" s="6">
-        <v>45863</v>
+        <v>45852</v>
       </c>
       <c r="H11" s="6">
-        <v>45863</v>
+        <v>45852</v>
       </c>
       <c r="I11" s="20">
         <v>0.755</v>
       </c>
       <c r="J11" s="21">
-        <v>0.34720000000000001</v>
+        <v>0.21879999999999999</v>
       </c>
       <c r="K11" s="9">
+        <v>10</v>
+      </c>
+      <c r="L11" s="22">
         <v>9</v>
       </c>
-      <c r="L11" s="22">
-        <v>13</v>
-      </c>
       <c r="M11" s="22">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="N11" s="22">
-        <v>13.5</v>
+        <v>11.5</v>
       </c>
       <c r="O11" s="22">
         <v>1</v>
@@ -1759,13 +1837,13 @@
       <c r="T11" s="27"/>
       <c r="U11" s="27"/>
       <c r="V11" s="1">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="W11" s="1">
+        <v>2</v>
+      </c>
+      <c r="X11" s="1">
         <v>1</v>
-      </c>
-      <c r="X11" s="1">
-        <v>2</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
@@ -1782,37 +1860,37 @@
         <v>2043</v>
       </c>
       <c r="E12" s="1">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="F12" s="1">
-        <v>115404</v>
+        <v>111960</v>
       </c>
       <c r="G12" s="6">
-        <v>45986</v>
+        <v>45707</v>
       </c>
       <c r="H12" s="6">
-        <v>45986</v>
+        <v>45707</v>
       </c>
       <c r="I12" s="20">
-        <v>0.755</v>
+        <v>0.80410000000000004</v>
       </c>
       <c r="J12" s="21">
-        <v>1</v>
+        <v>0.125</v>
       </c>
       <c r="K12" s="9">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="L12" s="22">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="M12" s="22">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="N12" s="22">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="O12" s="22">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P12" s="23"/>
       <c r="Q12" s="24"/>
@@ -1821,10 +1899,10 @@
       <c r="T12" s="27"/>
       <c r="U12" s="27"/>
       <c r="V12" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="W12" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="X12" s="1">
         <v>0</v>
@@ -1844,37 +1922,37 @@
         <v>2043</v>
       </c>
       <c r="E13" s="1">
-        <v>2692</v>
+        <v>2043</v>
       </c>
       <c r="F13" s="1">
-        <v>113450</v>
+        <v>113076</v>
       </c>
       <c r="G13" s="6">
-        <v>45852</v>
+        <v>45806</v>
       </c>
       <c r="H13" s="6">
-        <v>45852</v>
+        <v>45806</v>
       </c>
       <c r="I13" s="20">
         <v>0.755</v>
       </c>
       <c r="J13" s="21">
-        <v>0.29170000000000001</v>
+        <v>1</v>
       </c>
       <c r="K13" s="9">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L13" s="22">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="M13" s="22">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="N13" s="22">
-        <v>11.5</v>
+        <v>10.5</v>
       </c>
       <c r="O13" s="22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P13" s="23"/>
       <c r="Q13" s="24"/>
@@ -1883,13 +1961,13 @@
       <c r="T13" s="27"/>
       <c r="U13" s="27"/>
       <c r="V13" s="1">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="W13" s="1">
         <v>2</v>
       </c>
       <c r="X13" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.2">
@@ -1906,37 +1984,37 @@
         <v>2043</v>
       </c>
       <c r="E14" s="1">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="F14" s="1">
-        <v>111960</v>
+        <v>112083</v>
       </c>
       <c r="G14" s="6">
-        <v>45707</v>
+        <v>45736</v>
       </c>
       <c r="H14" s="6">
-        <v>45707</v>
+        <v>45736</v>
       </c>
       <c r="I14" s="20">
-        <v>0.80410000000000004</v>
+        <v>1</v>
       </c>
       <c r="J14" s="21">
-        <v>0.1583</v>
+        <v>1</v>
       </c>
       <c r="K14" s="9">
         <v>14</v>
       </c>
       <c r="L14" s="22">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="M14" s="22">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="N14" s="22">
-        <v>11.5</v>
+        <v>10</v>
       </c>
       <c r="O14" s="22">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P14" s="23"/>
       <c r="Q14" s="24"/>
@@ -1945,13 +2023,13 @@
       <c r="T14" s="27"/>
       <c r="U14" s="27"/>
       <c r="V14" s="1">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="W14" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>0</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
@@ -1971,34 +2049,34 @@
         <v>2043</v>
       </c>
       <c r="F15" s="1">
-        <v>113076</v>
+        <v>114157</v>
       </c>
       <c r="G15" s="6">
-        <v>45806</v>
+        <v>45904</v>
       </c>
       <c r="H15" s="6">
-        <v>45806</v>
+        <v>45904</v>
       </c>
       <c r="I15" s="20">
         <v>0.755</v>
       </c>
       <c r="J15" s="21">
+        <v>0.22220000000000001</v>
+      </c>
+      <c r="K15" s="9">
+        <v>8</v>
+      </c>
+      <c r="L15" s="22">
+        <v>8</v>
+      </c>
+      <c r="M15" s="22">
         <v>1</v>
       </c>
-      <c r="K15" s="9">
-        <v>11</v>
-      </c>
-      <c r="L15" s="22">
-        <v>7</v>
-      </c>
-      <c r="M15" s="22">
-        <v>3.5</v>
-      </c>
       <c r="N15" s="22">
-        <v>10.5</v>
+        <v>9</v>
       </c>
       <c r="O15" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P15" s="23"/>
       <c r="Q15" s="24"/>
@@ -2007,13 +2085,13 @@
       <c r="T15" s="27"/>
       <c r="U15" s="27"/>
       <c r="V15" s="1">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="W15" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X15" s="1">
-        <v>1.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
@@ -2030,37 +2108,37 @@
         <v>2043</v>
       </c>
       <c r="E16" s="1">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="F16" s="1">
-        <v>114157</v>
+        <v>116060</v>
       </c>
       <c r="G16" s="6">
-        <v>45904</v>
+        <v>46010</v>
       </c>
       <c r="H16" s="6">
-        <v>45904</v>
+        <v>46010</v>
       </c>
       <c r="I16" s="20">
         <v>0.755</v>
       </c>
       <c r="J16" s="21">
-        <v>0.22220000000000001</v>
+        <v>1</v>
       </c>
       <c r="K16" s="9">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L16" s="22">
         <v>8</v>
       </c>
       <c r="M16" s="22">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N16" s="22">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="O16" s="22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P16" s="23"/>
       <c r="Q16" s="24"/>
@@ -2072,10 +2150,10 @@
         <v>6</v>
       </c>
       <c r="W16" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X16" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
@@ -2095,34 +2173,34 @@
         <v>2043</v>
       </c>
       <c r="F17" s="1">
-        <v>112083</v>
+        <v>114431</v>
       </c>
       <c r="G17" s="6">
-        <v>45736</v>
+        <v>45930</v>
       </c>
       <c r="H17" s="6">
-        <v>45736</v>
+        <v>45930</v>
       </c>
       <c r="I17" s="20">
-        <v>1</v>
+        <v>0.755</v>
       </c>
       <c r="J17" s="21">
-        <v>1</v>
+        <v>0.125</v>
       </c>
       <c r="K17" s="9">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="L17" s="22">
         <v>6</v>
       </c>
       <c r="M17" s="22">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="N17" s="22">
-        <v>9</v>
+        <v>6.5</v>
       </c>
       <c r="O17" s="22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P17" s="23"/>
       <c r="Q17" s="24"/>
@@ -2131,13 +2209,13 @@
       <c r="T17" s="27"/>
       <c r="U17" s="27"/>
       <c r="V17" s="1">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="W17" s="1">
+        <v>2</v>
+      </c>
+      <c r="X17" s="1">
         <v>0</v>
-      </c>
-      <c r="X17" s="1">
-        <v>1.5</v>
       </c>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.2">
@@ -2157,13 +2235,13 @@
         <v>2856</v>
       </c>
       <c r="F18" s="1">
-        <v>116060</v>
+        <v>112522</v>
       </c>
       <c r="G18" s="6">
-        <v>46010</v>
+        <v>45776</v>
       </c>
       <c r="H18" s="6">
-        <v>46010</v>
+        <v>45776</v>
       </c>
       <c r="I18" s="20">
         <v>0.755</v>
@@ -2172,16 +2250,16 @@
         <v>1</v>
       </c>
       <c r="K18" s="9">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="L18" s="22">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M18" s="22">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="N18" s="22">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="O18" s="22">
         <v>0</v>
@@ -2193,13 +2271,13 @@
       <c r="T18" s="27"/>
       <c r="U18" s="27"/>
       <c r="V18" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W18" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X18" s="1">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
@@ -2216,37 +2294,37 @@
         <v>2043</v>
       </c>
       <c r="E19" s="1">
-        <v>2692</v>
+        <v>2856</v>
       </c>
       <c r="F19" s="1">
-        <v>114431</v>
+        <v>116883</v>
       </c>
       <c r="G19" s="6">
-        <v>45930</v>
+        <v>46126</v>
       </c>
       <c r="H19" s="6">
-        <v>45930</v>
+        <v>46023</v>
       </c>
       <c r="I19" s="20">
-        <v>0.755</v>
+        <v>0</v>
       </c>
       <c r="J19" s="21">
-        <v>0.15279999999999999</v>
+        <v>1</v>
       </c>
       <c r="K19" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="L19" s="22">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M19" s="22">
         <v>0.5</v>
       </c>
       <c r="N19" s="22">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="O19" s="22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P19" s="23"/>
       <c r="Q19" s="24"/>
@@ -2255,13 +2333,13 @@
       <c r="T19" s="27"/>
       <c r="U19" s="27"/>
       <c r="V19" s="1">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
       <c r="W19" s="1">
         <v>2</v>
       </c>
       <c r="X19" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.2">
@@ -2281,13 +2359,13 @@
         <v>2856</v>
       </c>
       <c r="F20" s="1">
-        <v>112522</v>
+        <v>116876</v>
       </c>
       <c r="G20" s="6">
-        <v>45776</v>
+        <v>46111</v>
       </c>
       <c r="H20" s="6">
-        <v>45776</v>
+        <v>46111</v>
       </c>
       <c r="I20" s="20">
         <v>0.755</v>
@@ -2296,16 +2374,16 @@
         <v>1</v>
       </c>
       <c r="K20" s="9">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="L20" s="22">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="M20" s="22">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N20" s="22">
-        <v>6</v>
+        <v>4.5</v>
       </c>
       <c r="O20" s="22">
         <v>0</v>
@@ -2317,102 +2395,40 @@
       <c r="T20" s="27"/>
       <c r="U20" s="27"/>
       <c r="V20" s="1">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="W20" s="1">
         <v>0</v>
       </c>
       <c r="X20" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="1">
-        <v>2043</v>
-      </c>
-      <c r="E21" s="1">
-        <v>2856</v>
-      </c>
-      <c r="F21" s="1">
-        <v>116876</v>
-      </c>
-      <c r="G21" s="6">
-        <v>46111</v>
-      </c>
-      <c r="H21" s="6">
-        <v>46111</v>
-      </c>
-      <c r="I21" s="20">
-        <v>0.755</v>
-      </c>
-      <c r="J21" s="21">
-        <v>1</v>
-      </c>
-      <c r="K21" s="9">
-        <v>1</v>
-      </c>
-      <c r="L21" s="22">
-        <v>4</v>
-      </c>
-      <c r="M21" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N21" s="22">
-        <v>4.5</v>
-      </c>
-      <c r="O21" s="22">
-        <v>0</v>
-      </c>
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="22"/>
+      <c r="N21" s="22"/>
+      <c r="O21" s="22"/>
       <c r="P21" s="23"/>
       <c r="Q21" s="24"/>
       <c r="R21" s="23"/>
       <c r="S21" s="27"/>
       <c r="T21" s="27"/>
       <c r="U21" s="27"/>
-      <c r="V21" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="W21" s="1">
-        <v>0</v>
-      </c>
-      <c r="X21" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="20"/>
-      <c r="J22" s="21"/>
-      <c r="K22" s="9"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="22"/>
-      <c r="P22" s="23"/>
-      <c r="Q22" s="24"/>
-      <c r="R22" s="23"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
-      <c r="U22" s="27"/>
-      <c r="V22" s="1"/>
-      <c r="W22" s="1"/>
-      <c r="X22" s="1"/>
+      <c r="V21" s="1"/>
+      <c r="W21" s="1"/>
+      <c r="X21" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2420,44 +2436,69 @@
     <mergeCell ref="P3:U3"/>
     <mergeCell ref="L3:N3"/>
   </mergeCells>
-  <conditionalFormatting sqref="A6:K22 U6:U22">
+  <conditionalFormatting sqref="A21:X21">
+    <cfRule type="expression" dxfId="10" priority="16" stopIfTrue="1">
+      <formula>$B21&lt;&gt;""</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I21">
+    <cfRule type="expression" dxfId="9" priority="15" stopIfTrue="1">
+      <formula>AND($B21&lt;&gt;"",$L21&lt;0.85)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V21">
+    <cfRule type="expression" dxfId="8" priority="13" stopIfTrue="1">
+      <formula>AND($B21&lt;&gt;"",$Z21&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W21">
+    <cfRule type="expression" dxfId="7" priority="12" stopIfTrue="1">
+      <formula>AND($B21&lt;&gt;"",$AA21&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X21">
+    <cfRule type="expression" priority="11" stopIfTrue="1">
+      <formula>AND($B21&lt;&gt;"",$AB21&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A20:K20 U6:U20 A6:K19">
     <cfRule type="expression" dxfId="6" priority="8" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I22">
+  <conditionalFormatting sqref="I6:I20">
     <cfRule type="expression" dxfId="5" priority="7" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$L6&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J6:J22">
-    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
-      <formula>AND($B6&lt;&gt;"",$M$29&lt;0.85)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L6:T22">
-    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
+  <conditionalFormatting sqref="L6:T20">
+    <cfRule type="expression" dxfId="4" priority="2" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:V22">
-    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
+  <conditionalFormatting sqref="V6:V20">
+    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$Z6&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:X22">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="V6:X20">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W6:W22">
-    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="W6:W20">
+    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$AA6&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X6:X22">
+  <conditionalFormatting sqref="X6:X20">
     <cfRule type="expression" priority="3" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$AB6&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6:J21">
+    <cfRule type="expression" dxfId="0" priority="20" stopIfTrue="1">
+      <formula>AND($B6&lt;&gt;"",$M$28&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-04-29 10:46)
</commit_message>
<xml_diff>
--- a/camino_cumbre/CAMINO A LA CUMBRE.xlsx
+++ b/camino_cumbre/CAMINO A LA CUMBRE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/camino_cumbre/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82901A5-2E36-4B4D-A96F-E1B46BF06FA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD638B59-B277-174D-AEA5-2BF4B3035D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-720" yWindow="700" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
+    <workbookView xWindow="540" yWindow="1120" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -161,7 +161,7 @@
     <t>Pólizas Pagadas</t>
   </si>
   <si>
-    <t>Avance  al 17 de abril de 2026.</t>
+    <t>Avance  al 24 de abril de 2026.</t>
   </si>
 </sst>
 </file>
@@ -501,7 +501,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{5777CE91-9B5C-AD4F-B1FB-47F4B57F6892}"/>
     <cellStyle name="Porcentaje 2" xfId="2" xr:uid="{7B24C14E-EE44-314E-8590-6F0AEF4F900D}"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="33">
     <dxf>
       <border>
         <left style="hair">
@@ -691,6 +691,29 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -1008,7 +1031,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X21" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X21" totalsRowShown="0" headerRowDxfId="32" headerRowBorderDxfId="31" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
   <autoFilter ref="A4:X21" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}"/>
   <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{452BBEC3-C02A-954A-AF30-AAC8D4135219}" name="Dir. de Venta" dataCellStyle="Normal 2"/>
@@ -1017,21 +1040,21 @@
     <tableColumn id="4" xr3:uid="{E64AD030-9FFA-1B49-B7F8-31458F00EB96}" name="Mat" dataCellStyle="Normal 2"/>
     <tableColumn id="5" xr3:uid="{407858BC-0878-5E44-A050-843285231653}" name="Suc" dataCellStyle="Normal 2"/>
     <tableColumn id="6" xr3:uid="{6FEB1162-A9E3-244F-886A-8D5C735D8BE4}" name="Asesor" dataCellStyle="Normal 2"/>
-    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="29" dataCellStyle="Normal 2"/>
-    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="28" dataCellStyle="Normal 2"/>
-    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="27" dataCellStyle="Porcentaje 2"/>
-    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="26" dataCellStyle="Normal 2"/>
-    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="25" dataCellStyle="Normal 2"/>
-    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="24" dataCellStyle="Normal 2"/>
-    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="23" dataCellStyle="Normal 2"/>
-    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="22" dataCellStyle="Normal 2"/>
-    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="21" dataCellStyle="Normal 2"/>
-    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="20" dataCellStyle="Normal 2"/>
-    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="19" dataCellStyle="Normal 2"/>
-    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="18" dataCellStyle="Normal 2"/>
-    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="17" dataCellStyle="Normal 2"/>
-    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="16" dataCellStyle="Normal 2"/>
-    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="15" dataCellStyle="Normal 2"/>
+    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="30" dataCellStyle="Normal 2"/>
+    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="29" dataCellStyle="Normal 2"/>
+    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="28" dataCellStyle="Porcentaje 2"/>
+    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="27" dataCellStyle="Normal 2"/>
+    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="26" dataCellStyle="Normal 2"/>
+    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="25" dataCellStyle="Normal 2"/>
+    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="24" dataCellStyle="Normal 2"/>
+    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="23" dataCellStyle="Normal 2"/>
+    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="22" dataCellStyle="Normal 2"/>
+    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="21" dataCellStyle="Normal 2"/>
+    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="20" dataCellStyle="Normal 2"/>
+    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="19" dataCellStyle="Normal 2"/>
+    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="18" dataCellStyle="Normal 2"/>
+    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="17" dataCellStyle="Normal 2"/>
+    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="16" dataCellStyle="Normal 2"/>
     <tableColumn id="22" xr3:uid="{FB6CEF72-668C-CB49-ACCA-75A997C036A1}" name="Mes 1" dataCellStyle="Normal 2"/>
     <tableColumn id="23" xr3:uid="{58B1F16B-3FBB-3D4C-8C16-DD05D985324B}" name="Mes 2" dataCellStyle="Normal 2"/>
     <tableColumn id="24" xr3:uid="{B5A4E59E-794B-AB4B-BB2B-840B78865464}" name="Mes 3" dataCellStyle="Normal 2"/>
@@ -1571,7 +1594,7 @@
         <v>45600</v>
       </c>
       <c r="I6" s="20">
-        <v>0.99539999999999995</v>
+        <v>0.99590000000000001</v>
       </c>
       <c r="J6" s="21">
         <v>1</v>
@@ -1580,13 +1603,13 @@
         <v>18</v>
       </c>
       <c r="L6" s="22">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M6" s="22">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="N6" s="22">
-        <v>51</v>
+        <v>52.5</v>
       </c>
       <c r="O6" s="22">
         <v>0</v>
@@ -1633,22 +1656,22 @@
         <v>45639</v>
       </c>
       <c r="I7" s="20">
-        <v>0.95199999999999996</v>
+        <v>0.96850000000000003</v>
       </c>
       <c r="J7" s="21">
-        <v>0.32640000000000002</v>
+        <v>0.34720000000000001</v>
       </c>
       <c r="K7" s="9">
         <v>17</v>
       </c>
       <c r="L7" s="22">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="M7" s="22">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="N7" s="22">
-        <v>24.5</v>
+        <v>26</v>
       </c>
       <c r="O7" s="22">
         <v>1</v>
@@ -1943,7 +1966,7 @@
         <v>45707</v>
       </c>
       <c r="I12" s="20">
-        <v>0.80410000000000004</v>
+        <v>0.755</v>
       </c>
       <c r="J12" s="21">
         <v>0.125</v>
@@ -2315,7 +2338,7 @@
         <v>45776</v>
       </c>
       <c r="I18" s="20">
-        <v>0.755</v>
+        <v>0.80589999999999995</v>
       </c>
       <c r="J18" s="21">
         <v>1</v>
@@ -2377,7 +2400,7 @@
         <v>46126</v>
       </c>
       <c r="I19" s="20">
-        <v>0</v>
+        <v>0.755</v>
       </c>
       <c r="J19" s="21">
         <v>1</v>
@@ -2508,17 +2531,17 @@
     <mergeCell ref="L3:N3"/>
   </mergeCells>
   <conditionalFormatting sqref="A21:X21">
-    <cfRule type="expression" dxfId="13" priority="24" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="32" stopIfTrue="1">
       <formula>$B21&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I21">
-    <cfRule type="expression" dxfId="12" priority="15" stopIfTrue="1">
+    <cfRule type="expression" dxfId="13" priority="15" stopIfTrue="1">
       <formula>AND($B21&lt;&gt;"",$L21&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J21">
-    <cfRule type="expression" dxfId="11" priority="28" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="36" stopIfTrue="1">
       <formula>AND($B21&lt;&gt;"",$M$28&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-11 13:33)
</commit_message>
<xml_diff>
--- a/camino_cumbre/CAMINO A LA CUMBRE.xlsx
+++ b/camino_cumbre/CAMINO A LA CUMBRE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/camino_cumbre/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD638B59-B277-174D-AEA5-2BF4B3035D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBB5356E-4DFC-1046-95E5-2102B151E694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="540" yWindow="1120" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
+    <workbookView xWindow="1680" yWindow="840" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -161,7 +161,7 @@
     <t>Pólizas Pagadas</t>
   </si>
   <si>
-    <t>Avance  al 24 de abril de 2026.</t>
+    <t>Avance  al 30 de abril de 2026.</t>
   </si>
 </sst>
 </file>
@@ -1603,13 +1603,13 @@
         <v>18</v>
       </c>
       <c r="L6" s="22">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M6" s="22">
         <v>4.5</v>
       </c>
       <c r="N6" s="22">
-        <v>52.5</v>
+        <v>53.5</v>
       </c>
       <c r="O6" s="22">
         <v>0</v>
@@ -1783,19 +1783,19 @@
         <v>0.755</v>
       </c>
       <c r="J9" s="21">
-        <v>0.26040000000000002</v>
+        <v>0.28129999999999999</v>
       </c>
       <c r="K9" s="9">
         <v>10</v>
       </c>
       <c r="L9" s="22">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M9" s="22">
         <v>0.5</v>
       </c>
       <c r="N9" s="22">
-        <v>13.5</v>
+        <v>14.5</v>
       </c>
       <c r="O9" s="22">
         <v>1</v>
@@ -2264,37 +2264,37 @@
         <v>2043</v>
       </c>
       <c r="E17" s="1">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="F17" s="1">
-        <v>114431</v>
+        <v>116883</v>
       </c>
       <c r="G17" s="6">
-        <v>45930</v>
+        <v>46126</v>
       </c>
       <c r="H17" s="6">
-        <v>45930</v>
+        <v>46126</v>
       </c>
       <c r="I17" s="20">
         <v>0.755</v>
       </c>
       <c r="J17" s="21">
-        <v>9.7199999999999995E-2</v>
+        <v>1</v>
       </c>
       <c r="K17" s="9">
+        <v>1</v>
+      </c>
+      <c r="L17" s="22">
+        <v>7</v>
+      </c>
+      <c r="M17" s="22">
+        <v>1</v>
+      </c>
+      <c r="N17" s="22">
         <v>8</v>
       </c>
-      <c r="L17" s="22">
-        <v>6</v>
-      </c>
-      <c r="M17" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N17" s="22">
-        <v>6.5</v>
-      </c>
       <c r="O17" s="22">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="P17" s="23"/>
       <c r="Q17" s="24"/>
@@ -2303,10 +2303,10 @@
       <c r="T17" s="27"/>
       <c r="U17" s="27"/>
       <c r="V17" s="1">
-        <v>4.5</v>
+        <v>8</v>
       </c>
       <c r="W17" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X17" s="1">
         <v>0</v>
@@ -2326,37 +2326,37 @@
         <v>2043</v>
       </c>
       <c r="E18" s="1">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="F18" s="1">
-        <v>112522</v>
+        <v>114431</v>
       </c>
       <c r="G18" s="6">
-        <v>45776</v>
+        <v>45930</v>
       </c>
       <c r="H18" s="6">
-        <v>45776</v>
+        <v>45930</v>
       </c>
       <c r="I18" s="20">
-        <v>0.80589999999999995</v>
+        <v>0.755</v>
       </c>
       <c r="J18" s="21">
-        <v>1</v>
+        <v>9.7199999999999995E-2</v>
       </c>
       <c r="K18" s="9">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="L18" s="22">
         <v>6</v>
       </c>
       <c r="M18" s="22">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N18" s="22">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="O18" s="22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P18" s="23"/>
       <c r="Q18" s="24"/>
@@ -2365,13 +2365,13 @@
       <c r="T18" s="27"/>
       <c r="U18" s="27"/>
       <c r="V18" s="1">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="W18" s="1">
+        <v>2</v>
+      </c>
+      <c r="X18" s="1">
         <v>0</v>
-      </c>
-      <c r="X18" s="1">
-        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.2">
@@ -2391,31 +2391,31 @@
         <v>2856</v>
       </c>
       <c r="F19" s="1">
-        <v>116883</v>
+        <v>112522</v>
       </c>
       <c r="G19" s="6">
-        <v>46126</v>
+        <v>45776</v>
       </c>
       <c r="H19" s="6">
-        <v>46126</v>
+        <v>45776</v>
       </c>
       <c r="I19" s="20">
-        <v>0.755</v>
+        <v>0.80589999999999995</v>
       </c>
       <c r="J19" s="21">
         <v>1</v>
       </c>
       <c r="K19" s="9">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="L19" s="22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M19" s="22">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="N19" s="22">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="O19" s="22">
         <v>0</v>
@@ -2427,13 +2427,13 @@
       <c r="T19" s="27"/>
       <c r="U19" s="27"/>
       <c r="V19" s="1">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="W19" s="1">
         <v>0</v>
       </c>
       <c r="X19" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:24" x14ac:dyDescent="0.2">
@@ -2531,7 +2531,7 @@
     <mergeCell ref="L3:N3"/>
   </mergeCells>
   <conditionalFormatting sqref="A21:X21">
-    <cfRule type="expression" dxfId="14" priority="32" stopIfTrue="1">
+    <cfRule type="expression" dxfId="14" priority="40" stopIfTrue="1">
       <formula>$B21&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2541,7 +2541,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J21">
-    <cfRule type="expression" dxfId="11" priority="36" stopIfTrue="1">
+    <cfRule type="expression" dxfId="11" priority="44" stopIfTrue="1">
       <formula>AND($B21&lt;&gt;"",$M$28&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
data: Actualización automática de reportes (2026-05-26 10:52)
</commit_message>
<xml_diff>
--- a/camino_cumbre/CAMINO A LA CUMBRE.xlsx
+++ b/camino_cumbre/CAMINO A LA CUMBRE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/camino_cumbre/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBB5356E-4DFC-1046-95E5-2102B151E694}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60726726-5350-5A45-A52D-206E5D071207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="840" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
+    <workbookView xWindow="4340" yWindow="840" windowWidth="24460" windowHeight="15320" xr2:uid="{745E7AD5-B7FE-F04B-8E22-39A4084D2BAB}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="42">
   <si>
     <t>Dir. de Venta</t>
   </si>
@@ -161,7 +161,7 @@
     <t>Pólizas Pagadas</t>
   </si>
   <si>
-    <t>Avance  al 30 de abril de 2026.</t>
+    <t>Avance  al 20 de Mayo de 2026.</t>
   </si>
 </sst>
 </file>
@@ -501,39 +501,7 @@
     <cellStyle name="Normal 2" xfId="1" xr:uid="{5777CE91-9B5C-AD4F-B1FB-47F4B57F6892}"/>
     <cellStyle name="Porcentaje 2" xfId="2" xr:uid="{7B24C14E-EE44-314E-8590-6F0AEF4F900D}"/>
   </cellStyles>
-  <dxfs count="33">
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="29">
     <dxf>
       <font>
         <b/>
@@ -574,6 +542,22 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -597,6 +581,22 @@
       </border>
     </dxf>
     <dxf>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -652,22 +652,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -691,22 +675,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -737,45 +705,6 @@
         <extend val="0"/>
         <color indexed="10"/>
       </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -1031,8 +960,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X21" totalsRowShown="0" headerRowDxfId="32" headerRowBorderDxfId="31" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
-  <autoFilter ref="A4:X21" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}" name="Tabla2" displayName="Tabla2" ref="A4:X18" totalsRowShown="0" headerRowDxfId="28" headerRowBorderDxfId="27" headerRowCellStyle="Normal 2" dataCellStyle="Normal 2">
+  <autoFilter ref="A4:X18" xr:uid="{578E9E09-B2CB-F649-A137-7A03C1727CDF}"/>
   <tableColumns count="24">
     <tableColumn id="1" xr3:uid="{452BBEC3-C02A-954A-AF30-AAC8D4135219}" name="Dir. de Venta" dataCellStyle="Normal 2"/>
     <tableColumn id="2" xr3:uid="{96963370-19D6-F44C-A2DA-2A40ED43DD5C}" name="Oficina" dataCellStyle="Normal 2"/>
@@ -1040,21 +969,21 @@
     <tableColumn id="4" xr3:uid="{E64AD030-9FFA-1B49-B7F8-31458F00EB96}" name="Mat" dataCellStyle="Normal 2"/>
     <tableColumn id="5" xr3:uid="{407858BC-0878-5E44-A050-843285231653}" name="Suc" dataCellStyle="Normal 2"/>
     <tableColumn id="6" xr3:uid="{6FEB1162-A9E3-244F-886A-8D5C735D8BE4}" name="Asesor" dataCellStyle="Normal 2"/>
-    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="30" dataCellStyle="Normal 2"/>
-    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="29" dataCellStyle="Normal 2"/>
-    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="28" dataCellStyle="Porcentaje 2"/>
-    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="27" dataCellStyle="Normal 2"/>
-    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="26" dataCellStyle="Normal 2"/>
-    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="25" dataCellStyle="Normal 2"/>
-    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="24" dataCellStyle="Normal 2"/>
-    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="23" dataCellStyle="Normal 2"/>
-    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="22" dataCellStyle="Normal 2"/>
-    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="21" dataCellStyle="Normal 2"/>
-    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="20" dataCellStyle="Normal 2"/>
-    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="19" dataCellStyle="Normal 2"/>
-    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="18" dataCellStyle="Normal 2"/>
-    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="17" dataCellStyle="Normal 2"/>
-    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="16" dataCellStyle="Normal 2"/>
+    <tableColumn id="7" xr3:uid="{A6C47CB4-51A8-AC4A-8E8A-91F8EBC90FAF}" name="Conexión" dataDxfId="26" dataCellStyle="Normal 2"/>
+    <tableColumn id="8" xr3:uid="{13AEAA9B-5D80-7445-B715-1B9DEE371D57}" name="Concurso" dataDxfId="25" dataCellStyle="Normal 2"/>
+    <tableColumn id="9" xr3:uid="{8D48CCB9-6544-AE45-B2C5-C2D673C725C5}" name="LIMRA" dataDxfId="24" dataCellStyle="Porcentaje 2"/>
+    <tableColumn id="10" xr3:uid="{B2FAE362-4A75-AE49-9576-61E713815186}" name="% Pol. En Vigor" dataDxfId="23" dataCellStyle="Normal 2"/>
+    <tableColumn id="11" xr3:uid="{BBCB44D8-F891-B44B-8387-861CF6E9DF19}" name="Mes" dataDxfId="22" dataCellStyle="Normal 2"/>
+    <tableColumn id="12" xr3:uid="{8ABB3BE3-3E57-B847-8D1C-9662D0105D10}" name="Pólizas Vida" dataDxfId="21" dataCellStyle="Normal 2"/>
+    <tableColumn id="13" xr3:uid="{67EBA4D1-7301-6949-990F-F690B48E34D0}" name="Pólizas GMM" dataDxfId="20" dataCellStyle="Normal 2"/>
+    <tableColumn id="14" xr3:uid="{3A1087EB-0F1F-E843-AFBA-9715B422272F}" name="Total" dataDxfId="19" dataCellStyle="Normal 2"/>
+    <tableColumn id="15" xr3:uid="{70AAFF82-E0DC-7E47-A3DA-69D547B18ECC}" name="Pólizas Canceladas" dataDxfId="18" dataCellStyle="Normal 2"/>
+    <tableColumn id="16" xr3:uid="{38391235-6C97-994B-8807-7D97AE60C293}" name="Kubor" dataDxfId="17" dataCellStyle="Normal 2"/>
+    <tableColumn id="17" xr3:uid="{A2FAA114-FE57-CE48-9674-BC10B5A0E337}" name="Mont Blanc" dataDxfId="16" dataCellStyle="Normal 2"/>
+    <tableColumn id="18" xr3:uid="{A4A65314-C415-DE4B-A724-6E1157AFF898}" name="Elbrús" dataDxfId="15" dataCellStyle="Normal 2"/>
+    <tableColumn id="19" xr3:uid="{1040FE48-FA96-3A4E-8A51-7F55DE596689}" name="Mickinley" dataDxfId="14" dataCellStyle="Normal 2"/>
+    <tableColumn id="20" xr3:uid="{8DDE3CDF-2E9D-7B46-BB69-F7108DC8C68A}" name="Kilimanjaro" dataDxfId="13" dataCellStyle="Normal 2"/>
+    <tableColumn id="21" xr3:uid="{D2643CF2-E0B8-F94D-BCA1-4B858C9D01EB}" name="Everest" dataDxfId="12" dataCellStyle="Normal 2"/>
     <tableColumn id="22" xr3:uid="{FB6CEF72-668C-CB49-ACCA-75A997C036A1}" name="Mes 1" dataCellStyle="Normal 2"/>
     <tableColumn id="23" xr3:uid="{58B1F16B-3FBB-3D4C-8C16-DD05D985324B}" name="Mes 2" dataCellStyle="Normal 2"/>
     <tableColumn id="24" xr3:uid="{B5A4E59E-794B-AB4B-BB2B-840B78865464}" name="Mes 3" dataCellStyle="Normal 2"/>
@@ -1380,7 +1309,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54AB4B63-646E-974E-8074-72018385EA77}">
-  <dimension ref="A1:X21"/>
+  <dimension ref="A1:X18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
@@ -1541,7 +1470,7 @@
       </c>
       <c r="O5" s="15"/>
       <c r="P5" s="19">
-        <f t="shared" ref="P5:U5" si="0">COUNTIF(P6:P65512,"p")</f>
+        <f t="shared" ref="P5:U5" si="0">COUNTIF(P6:P65509,"p")</f>
         <v>0</v>
       </c>
       <c r="Q5" s="19">
@@ -1582,37 +1511,37 @@
         <v>2043</v>
       </c>
       <c r="E6" s="1">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="F6" s="1">
-        <v>110453</v>
+        <v>111056</v>
       </c>
       <c r="G6" s="6">
-        <v>45600</v>
+        <v>45639</v>
       </c>
       <c r="H6" s="6">
-        <v>45600</v>
+        <v>45639</v>
       </c>
       <c r="I6" s="20">
-        <v>0.99590000000000001</v>
+        <v>0.8145</v>
       </c>
       <c r="J6" s="21">
-        <v>1</v>
+        <v>0.31940000000000002</v>
       </c>
       <c r="K6" s="9">
         <v>18</v>
       </c>
       <c r="L6" s="22">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="M6" s="22">
-        <v>4.5</v>
+        <v>8</v>
       </c>
       <c r="N6" s="22">
-        <v>53.5</v>
+        <v>26</v>
       </c>
       <c r="O6" s="22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="P6" s="23"/>
       <c r="Q6" s="24"/>
@@ -1621,13 +1550,13 @@
       <c r="T6" s="27"/>
       <c r="U6" s="27"/>
       <c r="V6" s="1">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="W6" s="1">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="X6" s="1">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
@@ -1644,37 +1573,37 @@
         <v>2043</v>
       </c>
       <c r="E7" s="1">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="F7" s="1">
-        <v>111056</v>
+        <v>115047</v>
       </c>
       <c r="G7" s="6">
-        <v>45639</v>
+        <v>45944</v>
       </c>
       <c r="H7" s="6">
-        <v>45639</v>
+        <v>45944</v>
       </c>
       <c r="I7" s="20">
-        <v>0.96850000000000003</v>
+        <v>0.755</v>
       </c>
       <c r="J7" s="21">
-        <v>0.34720000000000001</v>
+        <v>1</v>
       </c>
       <c r="K7" s="9">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="L7" s="22">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="M7" s="22">
-        <v>8</v>
+        <v>1.5</v>
       </c>
       <c r="N7" s="22">
-        <v>26</v>
+        <v>14.5</v>
       </c>
       <c r="O7" s="22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P7" s="23"/>
       <c r="Q7" s="24"/>
@@ -1683,13 +1612,13 @@
       <c r="T7" s="27"/>
       <c r="U7" s="27"/>
       <c r="V7" s="1">
-        <v>8</v>
+        <v>8.5</v>
       </c>
       <c r="W7" s="1">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="X7" s="1">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
@@ -1709,34 +1638,34 @@
         <v>2856</v>
       </c>
       <c r="F8" s="1">
-        <v>115047</v>
+        <v>114100</v>
       </c>
       <c r="G8" s="6">
-        <v>45944</v>
+        <v>45863</v>
       </c>
       <c r="H8" s="6">
-        <v>45944</v>
+        <v>45863</v>
       </c>
       <c r="I8" s="20">
         <v>0.755</v>
       </c>
       <c r="J8" s="21">
-        <v>1</v>
+        <v>0.28129999999999999</v>
       </c>
       <c r="K8" s="9">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="L8" s="22">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M8" s="22">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="N8" s="22">
         <v>14.5</v>
       </c>
       <c r="O8" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" s="23"/>
       <c r="Q8" s="24"/>
@@ -1745,13 +1674,13 @@
       <c r="T8" s="27"/>
       <c r="U8" s="27"/>
       <c r="V8" s="1">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="W8" s="1">
+        <v>1</v>
+      </c>
+      <c r="X8" s="1">
         <v>2</v>
-      </c>
-      <c r="X8" s="1">
-        <v>1.5</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
@@ -1768,37 +1697,37 @@
         <v>2043</v>
       </c>
       <c r="E9" s="1">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="F9" s="1">
-        <v>114100</v>
+        <v>115404</v>
       </c>
       <c r="G9" s="6">
-        <v>45863</v>
+        <v>45986</v>
       </c>
       <c r="H9" s="6">
-        <v>45863</v>
+        <v>45986</v>
       </c>
       <c r="I9" s="20">
         <v>0.755</v>
       </c>
       <c r="J9" s="21">
-        <v>0.28129999999999999</v>
+        <v>1</v>
       </c>
       <c r="K9" s="9">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L9" s="22">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M9" s="22">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="N9" s="22">
-        <v>14.5</v>
+        <v>12</v>
       </c>
       <c r="O9" s="22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P9" s="23"/>
       <c r="Q9" s="24"/>
@@ -1807,13 +1736,13 @@
       <c r="T9" s="27"/>
       <c r="U9" s="27"/>
       <c r="V9" s="1">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="W9" s="1">
         <v>1</v>
       </c>
       <c r="X9" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.2">
@@ -1833,34 +1762,34 @@
         <v>2043</v>
       </c>
       <c r="F10" s="1">
-        <v>115404</v>
+        <v>113450</v>
       </c>
       <c r="G10" s="6">
-        <v>45986</v>
+        <v>45852</v>
       </c>
       <c r="H10" s="6">
-        <v>45986</v>
+        <v>45852</v>
       </c>
       <c r="I10" s="20">
         <v>0.755</v>
       </c>
       <c r="J10" s="21">
-        <v>1</v>
+        <v>0.21879999999999999</v>
       </c>
       <c r="K10" s="9">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="L10" s="22">
         <v>9</v>
       </c>
       <c r="M10" s="22">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="N10" s="22">
-        <v>12</v>
+        <v>11.5</v>
       </c>
       <c r="O10" s="22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P10" s="23"/>
       <c r="Q10" s="24"/>
@@ -1869,13 +1798,13 @@
       <c r="T10" s="27"/>
       <c r="U10" s="27"/>
       <c r="V10" s="1">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W10" s="1">
+        <v>2</v>
+      </c>
+      <c r="X10" s="1">
         <v>1</v>
-      </c>
-      <c r="X10" s="1">
-        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.2">
@@ -1895,34 +1824,34 @@
         <v>2043</v>
       </c>
       <c r="F11" s="1">
-        <v>113450</v>
+        <v>112083</v>
       </c>
       <c r="G11" s="6">
-        <v>45852</v>
+        <v>45736</v>
       </c>
       <c r="H11" s="6">
-        <v>45852</v>
+        <v>45736</v>
       </c>
       <c r="I11" s="20">
-        <v>0.755</v>
+        <v>1</v>
       </c>
       <c r="J11" s="21">
-        <v>0.21879999999999999</v>
+        <v>1</v>
       </c>
       <c r="K11" s="9">
+        <v>15</v>
+      </c>
+      <c r="L11" s="22">
+        <v>7</v>
+      </c>
+      <c r="M11" s="22">
+        <v>3</v>
+      </c>
+      <c r="N11" s="22">
         <v>10</v>
       </c>
-      <c r="L11" s="22">
-        <v>9</v>
-      </c>
-      <c r="M11" s="22">
-        <v>2.5</v>
-      </c>
-      <c r="N11" s="22">
-        <v>11.5</v>
-      </c>
       <c r="O11" s="22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P11" s="23"/>
       <c r="Q11" s="24"/>
@@ -1931,13 +1860,13 @@
       <c r="T11" s="27"/>
       <c r="U11" s="27"/>
       <c r="V11" s="1">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="W11" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>1</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.2">
@@ -1954,37 +1883,37 @@
         <v>2043</v>
       </c>
       <c r="E12" s="1">
-        <v>2856</v>
+        <v>2043</v>
       </c>
       <c r="F12" s="1">
-        <v>111960</v>
+        <v>114157</v>
       </c>
       <c r="G12" s="6">
-        <v>45707</v>
+        <v>45904</v>
       </c>
       <c r="H12" s="6">
-        <v>45707</v>
+        <v>45904</v>
       </c>
       <c r="I12" s="20">
         <v>0.755</v>
       </c>
       <c r="J12" s="21">
-        <v>0.125</v>
+        <v>0.2361</v>
       </c>
       <c r="K12" s="9">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="L12" s="22">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M12" s="22">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="N12" s="22">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="O12" s="22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="P12" s="23"/>
       <c r="Q12" s="24"/>
@@ -1996,10 +1925,10 @@
         <v>6</v>
       </c>
       <c r="W12" s="1">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.2">
@@ -2016,16 +1945,16 @@
         <v>2043</v>
       </c>
       <c r="E13" s="1">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="F13" s="1">
-        <v>113076</v>
+        <v>116060</v>
       </c>
       <c r="G13" s="6">
-        <v>45806</v>
+        <v>46010</v>
       </c>
       <c r="H13" s="6">
-        <v>45806</v>
+        <v>46010</v>
       </c>
       <c r="I13" s="20">
         <v>0.755</v>
@@ -2034,16 +1963,16 @@
         <v>1</v>
       </c>
       <c r="K13" s="9">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="L13" s="22">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M13" s="22">
-        <v>3.5</v>
+        <v>0.5</v>
       </c>
       <c r="N13" s="22">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="O13" s="22">
         <v>0</v>
@@ -2055,10 +1984,10 @@
       <c r="T13" s="27"/>
       <c r="U13" s="27"/>
       <c r="V13" s="1">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="W13" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X13" s="1">
         <v>1.5</v>
@@ -2078,34 +2007,34 @@
         <v>2043</v>
       </c>
       <c r="E14" s="1">
-        <v>2043</v>
+        <v>2856</v>
       </c>
       <c r="F14" s="1">
-        <v>112083</v>
+        <v>116883</v>
       </c>
       <c r="G14" s="6">
-        <v>45736</v>
+        <v>46126</v>
       </c>
       <c r="H14" s="6">
-        <v>45736</v>
+        <v>46126</v>
       </c>
       <c r="I14" s="20">
-        <v>1</v>
+        <v>0.755</v>
       </c>
       <c r="J14" s="21">
         <v>1</v>
       </c>
       <c r="K14" s="9">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="L14" s="22">
         <v>7</v>
       </c>
       <c r="M14" s="22">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N14" s="22">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O14" s="22">
         <v>0</v>
@@ -2117,13 +2046,13 @@
       <c r="T14" s="27"/>
       <c r="U14" s="27"/>
       <c r="V14" s="1">
-        <v>5.5</v>
+        <v>8</v>
       </c>
       <c r="W14" s="1">
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>1.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.2">
@@ -2143,34 +2072,34 @@
         <v>2043</v>
       </c>
       <c r="F15" s="1">
-        <v>114157</v>
+        <v>117440</v>
       </c>
       <c r="G15" s="6">
-        <v>45904</v>
+        <v>46149</v>
       </c>
       <c r="H15" s="6">
-        <v>45904</v>
+        <v>46149</v>
       </c>
       <c r="I15" s="20">
         <v>0.755</v>
       </c>
       <c r="J15" s="21">
-        <v>0.2361</v>
+        <v>1</v>
       </c>
       <c r="K15" s="9">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L15" s="22">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M15" s="22">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="N15" s="22">
-        <v>9.5</v>
+        <v>6</v>
       </c>
       <c r="O15" s="22">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P15" s="23"/>
       <c r="Q15" s="24"/>
@@ -2185,7 +2114,7 @@
         <v>0</v>
       </c>
       <c r="X15" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.2">
@@ -2205,31 +2134,31 @@
         <v>2856</v>
       </c>
       <c r="F16" s="1">
-        <v>116060</v>
+        <v>112522</v>
       </c>
       <c r="G16" s="6">
-        <v>46010</v>
+        <v>45776</v>
       </c>
       <c r="H16" s="6">
-        <v>46010</v>
+        <v>45776</v>
       </c>
       <c r="I16" s="20">
-        <v>0.755</v>
+        <v>0.80110000000000003</v>
       </c>
       <c r="J16" s="21">
         <v>1</v>
       </c>
       <c r="K16" s="9">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="L16" s="22">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M16" s="22">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="N16" s="22">
-        <v>8.5</v>
+        <v>6</v>
       </c>
       <c r="O16" s="22">
         <v>0</v>
@@ -2241,13 +2170,13 @@
       <c r="T16" s="27"/>
       <c r="U16" s="27"/>
       <c r="V16" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="W16" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X16" s="1">
-        <v>1.5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:24" x14ac:dyDescent="0.2">
@@ -2267,13 +2196,13 @@
         <v>2856</v>
       </c>
       <c r="F17" s="1">
-        <v>116883</v>
+        <v>116876</v>
       </c>
       <c r="G17" s="6">
-        <v>46126</v>
+        <v>46111</v>
       </c>
       <c r="H17" s="6">
-        <v>46126</v>
+        <v>46111</v>
       </c>
       <c r="I17" s="20">
         <v>0.755</v>
@@ -2282,16 +2211,16 @@
         <v>1</v>
       </c>
       <c r="K17" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L17" s="22">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M17" s="22">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N17" s="22">
-        <v>8</v>
+        <v>4.5</v>
       </c>
       <c r="O17" s="22">
         <v>0</v>
@@ -2303,7 +2232,7 @@
       <c r="T17" s="27"/>
       <c r="U17" s="27"/>
       <c r="V17" s="1">
-        <v>8</v>
+        <v>4.5</v>
       </c>
       <c r="W17" s="1">
         <v>0</v>
@@ -2313,216 +2242,30 @@
       </c>
     </row>
     <row r="18" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D18" s="1">
-        <v>2043</v>
-      </c>
-      <c r="E18" s="1">
-        <v>2043</v>
-      </c>
-      <c r="F18" s="1">
-        <v>114431</v>
-      </c>
-      <c r="G18" s="6">
-        <v>45930</v>
-      </c>
-      <c r="H18" s="6">
-        <v>45930</v>
-      </c>
-      <c r="I18" s="20">
-        <v>0.755</v>
-      </c>
-      <c r="J18" s="21">
-        <v>9.7199999999999995E-2</v>
-      </c>
-      <c r="K18" s="9">
-        <v>8</v>
-      </c>
-      <c r="L18" s="22">
-        <v>6</v>
-      </c>
-      <c r="M18" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N18" s="22">
-        <v>6.5</v>
-      </c>
-      <c r="O18" s="22">
-        <v>3</v>
-      </c>
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="20"/>
+      <c r="J18" s="21"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="22"/>
+      <c r="M18" s="22"/>
+      <c r="N18" s="22"/>
+      <c r="O18" s="22"/>
       <c r="P18" s="23"/>
       <c r="Q18" s="24"/>
       <c r="R18" s="23"/>
       <c r="S18" s="27"/>
       <c r="T18" s="27"/>
       <c r="U18" s="27"/>
-      <c r="V18" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="W18" s="1">
-        <v>2</v>
-      </c>
-      <c r="X18" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="1">
-        <v>2043</v>
-      </c>
-      <c r="E19" s="1">
-        <v>2856</v>
-      </c>
-      <c r="F19" s="1">
-        <v>112522</v>
-      </c>
-      <c r="G19" s="6">
-        <v>45776</v>
-      </c>
-      <c r="H19" s="6">
-        <v>45776</v>
-      </c>
-      <c r="I19" s="20">
-        <v>0.80589999999999995</v>
-      </c>
-      <c r="J19" s="21">
-        <v>1</v>
-      </c>
-      <c r="K19" s="9">
-        <v>13</v>
-      </c>
-      <c r="L19" s="22">
-        <v>6</v>
-      </c>
-      <c r="M19" s="22">
-        <v>0</v>
-      </c>
-      <c r="N19" s="22">
-        <v>6</v>
-      </c>
-      <c r="O19" s="22">
-        <v>0</v>
-      </c>
-      <c r="P19" s="23"/>
-      <c r="Q19" s="24"/>
-      <c r="R19" s="23"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
-      <c r="U19" s="27"/>
-      <c r="V19" s="1">
-        <v>4</v>
-      </c>
-      <c r="W19" s="1">
-        <v>0</v>
-      </c>
-      <c r="X19" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D20" s="1">
-        <v>2043</v>
-      </c>
-      <c r="E20" s="1">
-        <v>2856</v>
-      </c>
-      <c r="F20" s="1">
-        <v>116876</v>
-      </c>
-      <c r="G20" s="6">
-        <v>46111</v>
-      </c>
-      <c r="H20" s="6">
-        <v>46111</v>
-      </c>
-      <c r="I20" s="20">
-        <v>0.755</v>
-      </c>
-      <c r="J20" s="21">
-        <v>1</v>
-      </c>
-      <c r="K20" s="9">
-        <v>2</v>
-      </c>
-      <c r="L20" s="22">
-        <v>4</v>
-      </c>
-      <c r="M20" s="22">
-        <v>0.5</v>
-      </c>
-      <c r="N20" s="22">
-        <v>4.5</v>
-      </c>
-      <c r="O20" s="22">
-        <v>0</v>
-      </c>
-      <c r="P20" s="23"/>
-      <c r="Q20" s="24"/>
-      <c r="R20" s="23"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
-      <c r="U20" s="27"/>
-      <c r="V20" s="1">
-        <v>4.5</v>
-      </c>
-      <c r="W20" s="1">
-        <v>0</v>
-      </c>
-      <c r="X20" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1"/>
-      <c r="G21" s="6"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="9"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="22"/>
-      <c r="P21" s="23"/>
-      <c r="Q21" s="24"/>
-      <c r="R21" s="23"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
-      <c r="U21" s="27"/>
-      <c r="V21" s="1"/>
-      <c r="W21" s="1"/>
-      <c r="X21" s="1"/>
+      <c r="V18" s="1"/>
+      <c r="W18" s="1"/>
+      <c r="X18" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2530,74 +2273,74 @@
     <mergeCell ref="P3:U3"/>
     <mergeCell ref="L3:N3"/>
   </mergeCells>
-  <conditionalFormatting sqref="A21:X21">
-    <cfRule type="expression" dxfId="14" priority="40" stopIfTrue="1">
-      <formula>$B21&lt;&gt;""</formula>
+  <conditionalFormatting sqref="A18:X18">
+    <cfRule type="expression" dxfId="11" priority="48" stopIfTrue="1">
+      <formula>$B18&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I21">
-    <cfRule type="expression" dxfId="13" priority="15" stopIfTrue="1">
-      <formula>AND($B21&lt;&gt;"",$L21&lt;0.85)</formula>
+  <conditionalFormatting sqref="I18">
+    <cfRule type="expression" dxfId="10" priority="15" stopIfTrue="1">
+      <formula>AND($B18&lt;&gt;"",$L18&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J21">
-    <cfRule type="expression" dxfId="11" priority="44" stopIfTrue="1">
-      <formula>AND($B21&lt;&gt;"",$M$28&lt;0.85)</formula>
+  <conditionalFormatting sqref="J18">
+    <cfRule type="expression" dxfId="9" priority="52" stopIfTrue="1">
+      <formula>AND($B18&lt;&gt;"",$M$25&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V21">
-    <cfRule type="expression" dxfId="9" priority="13" stopIfTrue="1">
-      <formula>AND($B21&lt;&gt;"",$Z21&lt;1)</formula>
+  <conditionalFormatting sqref="V18">
+    <cfRule type="expression" dxfId="8" priority="13" stopIfTrue="1">
+      <formula>AND($B18&lt;&gt;"",$Z18&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W21">
+  <conditionalFormatting sqref="W18">
     <cfRule type="expression" dxfId="7" priority="12" stopIfTrue="1">
-      <formula>AND($B21&lt;&gt;"",$AA21&lt;1)</formula>
+      <formula>AND($B18&lt;&gt;"",$AA18&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X21">
+  <conditionalFormatting sqref="X18">
     <cfRule type="expression" priority="11" stopIfTrue="1">
-      <formula>AND($B21&lt;&gt;"",$AB21&lt;1)</formula>
+      <formula>AND($B18&lt;&gt;"",$AB18&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A20:K20 U6:U20 A6:K19">
+  <conditionalFormatting sqref="A17:K17 U6:U17 A6:K16">
     <cfRule type="expression" dxfId="6" priority="8" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I20">
+  <conditionalFormatting sqref="I6:I17">
     <cfRule type="expression" dxfId="5" priority="7" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$L6&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J6:J20">
-    <cfRule type="expression" dxfId="4" priority="6" stopIfTrue="1">
-      <formula>AND($B6&lt;&gt;"",$M$29&lt;0.85)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L6:T20">
-    <cfRule type="expression" dxfId="3" priority="2" stopIfTrue="1">
+  <conditionalFormatting sqref="L6:T17">
+    <cfRule type="expression" dxfId="4" priority="2" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:V20">
-    <cfRule type="expression" dxfId="2" priority="5" stopIfTrue="1">
+  <conditionalFormatting sqref="V6:V17">
+    <cfRule type="expression" dxfId="3" priority="5" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$Z6&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V6:X20">
-    <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
+  <conditionalFormatting sqref="V6:X17">
+    <cfRule type="expression" dxfId="2" priority="1" stopIfTrue="1">
       <formula>$B6&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W6:W20">
-    <cfRule type="expression" dxfId="0" priority="4" stopIfTrue="1">
+  <conditionalFormatting sqref="W6:W17">
+    <cfRule type="expression" dxfId="1" priority="4" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$AA6&lt;1)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X6:X20">
+  <conditionalFormatting sqref="X6:X17">
     <cfRule type="expression" priority="3" stopIfTrue="1">
       <formula>AND($B6&lt;&gt;"",$AB6&lt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J6:J17">
+    <cfRule type="expression" dxfId="0" priority="57" stopIfTrue="1">
+      <formula>AND($B6&lt;&gt;"",$M$26&lt;0.85)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>